<commit_message>
Excel switch ontology link and comment cols
</commit_message>
<xml_diff>
--- a/test/data/coincell_excel_schema.xlsx
+++ b/test/data/coincell_excel_schema.xlsx
@@ -523,8 +523,8 @@
     <col width="42" customWidth="1" min="2" max="2"/>
     <col width="9" customWidth="1" min="3" max="3"/>
     <col width="14" customWidth="1" min="4" max="4"/>
-    <col width="160" customWidth="1" min="5" max="5"/>
-    <col width="74" customWidth="1" min="6" max="6"/>
+    <col width="74" customWidth="1" min="5" max="5"/>
+    <col width="160" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1" ht="20" customHeight="1">
@@ -550,12 +550,12 @@
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
+          <t>Comment</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
           <t>Ontology link</t>
-        </is>
-      </c>
-      <c r="F1" s="1" t="inlineStr">
-        <is>
-          <t>Comment</t>
         </is>
       </c>
     </row>
@@ -594,12 +594,12 @@
       </c>
       <c r="E3" s="4" t="inlineStr">
         <is>
+          <t>Required, do not change</t>
+        </is>
+      </c>
+      <c r="F3" s="4" t="inlineStr">
+        <is>
           <t>type|</t>
-        </is>
-      </c>
-      <c r="F3" s="4" t="inlineStr">
-        <is>
-          <t>Required, do not change</t>
         </is>
       </c>
     </row>
@@ -626,12 +626,12 @@
       </c>
       <c r="E4" s="5" t="inlineStr">
         <is>
+          <t>Unique ID for cell</t>
+        </is>
+      </c>
+      <c r="F4" s="5" t="inlineStr">
+        <is>
           <t>schema:productID</t>
-        </is>
-      </c>
-      <c r="F4" s="5" t="inlineStr">
-        <is>
-          <t>Unique ID for cell</t>
         </is>
       </c>
     </row>
@@ -658,12 +658,12 @@
       </c>
       <c r="E5" s="4" t="inlineStr">
         <is>
+          <t>Human-friendly name for the cell</t>
+        </is>
+      </c>
+      <c r="F5" s="4" t="inlineStr">
+        <is>
           <t>schema:name</t>
-        </is>
-      </c>
-      <c r="F5" s="4" t="inlineStr">
-        <is>
-          <t>Human-friendly name for the cell</t>
         </is>
       </c>
     </row>
@@ -690,12 +690,12 @@
       </c>
       <c r="E6" s="5" t="inlineStr">
         <is>
+          <t>Assembly date in ISO8601 format (YYYY-MM-DD)</t>
+        </is>
+      </c>
+      <c r="F6" s="5" t="inlineStr">
+        <is>
           <t>schema:dateCreated</t>
-        </is>
-      </c>
-      <c r="F6" s="5" t="inlineStr">
-        <is>
-          <t>Assembly date in ISO8601 format (YYYY-MM-DD)</t>
         </is>
       </c>
     </row>
@@ -722,12 +722,12 @@
       </c>
       <c r="E7" s="4" t="inlineStr">
         <is>
+          <t>Organisation that made the cell, value should be in @classes with ID</t>
+        </is>
+      </c>
+      <c r="F7" s="4" t="inlineStr">
+        <is>
           <t>schema:manufacturer</t>
-        </is>
-      </c>
-      <c r="F7" s="4" t="inlineStr">
-        <is>
-          <t>Organisation that made the cell, value should be in @classes with ID</t>
         </is>
       </c>
     </row>
@@ -754,12 +754,12 @@
       </c>
       <c r="E8" s="5" t="inlineStr">
         <is>
+          <t>Person that made the cell, value should be in @classes with ID</t>
+        </is>
+      </c>
+      <c r="F8" s="5" t="inlineStr">
+        <is>
           <t>schema:creator</t>
-        </is>
-      </c>
-      <c r="F8" s="5" t="inlineStr">
-        <is>
-          <t>Person that made the cell, value should be in @classes with ID</t>
         </is>
       </c>
     </row>
@@ -784,12 +784,12 @@
           <t>recommended</t>
         </is>
       </c>
-      <c r="E9" s="4" t="inlineStr">
+      <c r="E9" s="4" t="n"/>
+      <c r="F9" s="4" t="inlineStr">
         <is>
           <t>rdfs:comment</t>
         </is>
       </c>
-      <c r="F9" s="4" t="n"/>
     </row>
     <row r="10">
       <c r="A10" s="5" t="inlineStr">
@@ -814,12 +814,12 @@
       </c>
       <c r="E10" s="5" t="inlineStr">
         <is>
+          <t>'manually' or 'by robot'</t>
+        </is>
+      </c>
+      <c r="F10" s="5" t="inlineStr">
+        <is>
           <t>rdfs:comment</t>
-        </is>
-      </c>
-      <c r="F10" s="5" t="inlineStr">
-        <is>
-          <t>'manually' or 'by robot'</t>
         </is>
       </c>
     </row>
@@ -846,12 +846,12 @@
       </c>
       <c r="E11" s="4" t="inlineStr">
         <is>
+          <t>Name of this schema, do not change</t>
+        </is>
+      </c>
+      <c r="F11" s="4" t="inlineStr">
+        <is>
           <t>rdfs:comment</t>
-        </is>
-      </c>
-      <c r="F11" s="4" t="inlineStr">
-        <is>
-          <t>Name of this schema, do not change</t>
         </is>
       </c>
     </row>
@@ -878,12 +878,12 @@
       </c>
       <c r="E12" s="5" t="inlineStr">
         <is>
+          <t>Version of this schema, do not change</t>
+        </is>
+      </c>
+      <c r="F12" s="5" t="inlineStr">
+        <is>
           <t>rdfs:comment</t>
-        </is>
-      </c>
-      <c r="F12" s="5" t="inlineStr">
-        <is>
-          <t>Version of this schema, do not change</t>
         </is>
       </c>
     </row>
@@ -920,12 +920,12 @@
           <t>required</t>
         </is>
       </c>
-      <c r="E14" s="4" t="inlineStr">
+      <c r="E14" s="4" t="n"/>
+      <c r="F14" s="4" t="inlineStr">
         <is>
           <t>hasPositiveElectrode-hasCurrentCollector</t>
         </is>
       </c>
-      <c r="F14" s="4" t="n"/>
     </row>
     <row r="15">
       <c r="A15" s="8" t="inlineStr">
@@ -946,12 +946,12 @@
           <t>recommended</t>
         </is>
       </c>
-      <c r="E15" s="8" t="inlineStr">
+      <c r="E15" s="8" t="n"/>
+      <c r="F15" s="8" t="inlineStr">
         <is>
           <t>hasPositiveElectrode-hasCurrentCollector-hasMeasuredProperty-Thickness</t>
         </is>
       </c>
-      <c r="F15" s="8" t="n"/>
     </row>
     <row r="16">
       <c r="A16" s="4" t="inlineStr">
@@ -974,12 +974,12 @@
           <t>required</t>
         </is>
       </c>
-      <c r="E16" s="4" t="inlineStr">
+      <c r="E16" s="4" t="n"/>
+      <c r="F16" s="4" t="inlineStr">
         <is>
           <t>hasPositiveElectrode-hasCoating-type|ElectrodeCoating-hasActiveMaterial</t>
         </is>
       </c>
-      <c r="F16" s="4" t="n"/>
     </row>
     <row r="17">
       <c r="A17" s="8" t="inlineStr">
@@ -1002,12 +1002,12 @@
           <t>recommended</t>
         </is>
       </c>
-      <c r="E17" s="8" t="inlineStr">
+      <c r="E17" s="8" t="n"/>
+      <c r="F17" s="8" t="inlineStr">
         <is>
           <t>hasPositiveElectrode-hasCoating-type|ElectrodeCoating-hasActiveMaterial-hasMeasuredProperty-type|molecularFormula-hasStringValue</t>
         </is>
       </c>
-      <c r="F17" s="8" t="n"/>
     </row>
     <row r="18">
       <c r="A18" s="4" t="inlineStr">
@@ -1028,12 +1028,12 @@
           <t>required</t>
         </is>
       </c>
-      <c r="E18" s="4" t="inlineStr">
+      <c r="E18" s="4" t="n"/>
+      <c r="F18" s="4" t="inlineStr">
         <is>
           <t>hasPositiveElectrode-hasCoating-type|ElectrodeCoating-hasActiveMaterial-hasMeasuredProperty-MassFraction</t>
         </is>
       </c>
-      <c r="F18" s="4" t="n"/>
     </row>
     <row r="19">
       <c r="A19" s="8" t="inlineStr">
@@ -1056,12 +1056,12 @@
           <t>required</t>
         </is>
       </c>
-      <c r="E19" s="8" t="inlineStr">
+      <c r="E19" s="8" t="n"/>
+      <c r="F19" s="8" t="inlineStr">
         <is>
           <t>hasPositiveElectrode-hasCoating-type|ElectrodeCoating-hasBinder</t>
         </is>
       </c>
-      <c r="F19" s="8" t="n"/>
     </row>
     <row r="20">
       <c r="A20" s="4" t="inlineStr">
@@ -1082,12 +1082,12 @@
           <t>required</t>
         </is>
       </c>
-      <c r="E20" s="4" t="inlineStr">
+      <c r="E20" s="4" t="n"/>
+      <c r="F20" s="4" t="inlineStr">
         <is>
           <t>hasPositiveElectrode-hasCoating-type|ElectrodeCoating-hasBinder-hasMeasuredProperty-MassFraction</t>
         </is>
       </c>
-      <c r="F20" s="4" t="n"/>
     </row>
     <row r="21">
       <c r="A21" s="8" t="inlineStr">
@@ -1110,12 +1110,12 @@
           <t>required</t>
         </is>
       </c>
-      <c r="E21" s="8" t="inlineStr">
+      <c r="E21" s="8" t="n"/>
+      <c r="F21" s="8" t="inlineStr">
         <is>
           <t>hasPositiveElectrode-hasCoating-type|ElectrodeCoating-hasConductiveAdditive</t>
         </is>
       </c>
-      <c r="F21" s="8" t="n"/>
     </row>
     <row r="22">
       <c r="A22" s="4" t="inlineStr">
@@ -1136,12 +1136,12 @@
           <t>required</t>
         </is>
       </c>
-      <c r="E22" s="4" t="inlineStr">
+      <c r="E22" s="4" t="n"/>
+      <c r="F22" s="4" t="inlineStr">
         <is>
           <t>hasPositiveElectrode-hasCoating-type|ElectrodeCoating-hasConductiveAdditive-hasMeasuredProperty-MassFraction</t>
         </is>
       </c>
-      <c r="F22" s="4" t="n"/>
     </row>
     <row r="23">
       <c r="A23" s="8" t="inlineStr">
@@ -1162,12 +1162,12 @@
           <t>required</t>
         </is>
       </c>
-      <c r="E23" s="8" t="inlineStr">
+      <c r="E23" s="8" t="n"/>
+      <c r="F23" s="8" t="inlineStr">
         <is>
           <t>hasPositiveElectrode-hasCoating-type|ElectrodeCoating-hasActiveMaterial-hasMeasuredProperty-MassLoading</t>
         </is>
       </c>
-      <c r="F23" s="8" t="n"/>
     </row>
     <row r="24">
       <c r="A24" s="4" t="inlineStr">
@@ -1188,12 +1188,12 @@
           <t>recommended</t>
         </is>
       </c>
-      <c r="E24" s="4" t="inlineStr">
+      <c r="E24" s="4" t="n"/>
+      <c r="F24" s="4" t="inlineStr">
         <is>
           <t>hasPositiveElectrode-hasCoating-type|ElectrodeCoating-hasMeasuredProperty-CalenderedCoatingThickness</t>
         </is>
       </c>
-      <c r="F24" s="4" t="n"/>
     </row>
     <row r="25">
       <c r="A25" s="9" t="inlineStr">
@@ -1226,12 +1226,12 @@
           <t>optional</t>
         </is>
       </c>
-      <c r="E26" s="4" t="inlineStr">
+      <c r="E26" s="4" t="n"/>
+      <c r="F26" s="4" t="inlineStr">
         <is>
           <t>hasPositiveElectrode-hasCoating-type|ElectrodeCoating-hasMeasuredProperty-Porosity</t>
         </is>
       </c>
-      <c r="F26" s="4" t="n"/>
     </row>
     <row r="27">
       <c r="A27" s="8" t="inlineStr">
@@ -1252,12 +1252,12 @@
           <t>optional</t>
         </is>
       </c>
-      <c r="E27" s="8" t="inlineStr">
+      <c r="E27" s="8" t="n"/>
+      <c r="F27" s="8" t="inlineStr">
         <is>
           <t>hasPositiveElectrode-hasCoating-type|ElectrodeCoating-hasMeasuredProperty-Tortuosity</t>
         </is>
       </c>
-      <c r="F27" s="8" t="n"/>
     </row>
     <row r="28">
       <c r="A28" s="4" t="inlineStr">
@@ -1278,12 +1278,12 @@
           <t>optional</t>
         </is>
       </c>
-      <c r="E28" s="4" t="inlineStr">
+      <c r="E28" s="4" t="n"/>
+      <c r="F28" s="4" t="inlineStr">
         <is>
           <t>hasPositiveElectrode-hasCoating-type|ElectrodeCoating-hasActiveMaterial-hasMeasuredProperty-D50ParticleSize</t>
         </is>
       </c>
-      <c r="F28" s="4" t="n"/>
     </row>
     <row r="29">
       <c r="A29" s="9" t="inlineStr">
@@ -1318,12 +1318,12 @@
           <t>optional</t>
         </is>
       </c>
-      <c r="E30" s="4" t="inlineStr">
+      <c r="E30" s="4" t="n"/>
+      <c r="F30" s="4" t="inlineStr">
         <is>
           <t>hasPositiveElectrode-hasMeasuredProperty-type|RatedCapacity-rev|hasOutput-type|Measurement-hasInput-ElectrochemicalHalfCell-rdfs:comment</t>
         </is>
       </c>
-      <c r="F30" s="4" t="n"/>
     </row>
     <row r="31">
       <c r="A31" s="8" t="inlineStr">
@@ -1346,12 +1346,12 @@
           <t>optional</t>
         </is>
       </c>
-      <c r="E31" s="8" t="inlineStr">
+      <c r="E31" s="8" t="n"/>
+      <c r="F31" s="8" t="inlineStr">
         <is>
           <t>hasPositiveElectrode-hasMeasuredProperty-type|RatedCapacity-rev|hasOutput-type|Measurement-hasInput-ElectrochemicalHalfCell-hasReferenceElectrode</t>
         </is>
       </c>
-      <c r="F31" s="8" t="n"/>
     </row>
     <row r="32">
       <c r="A32" s="4" t="inlineStr">
@@ -1372,12 +1372,12 @@
           <t>optional</t>
         </is>
       </c>
-      <c r="E32" s="4" t="inlineStr">
+      <c r="E32" s="4" t="n"/>
+      <c r="F32" s="4" t="inlineStr">
         <is>
           <t>hasPositiveElectrode-hasMeasuredProperty-type|RatedCapacity-rev|hasOutput-type|Measurement-hasInput-ConstantCurrentCharging-hasInput-LowerVoltageLimit</t>
         </is>
       </c>
-      <c r="F32" s="4" t="n"/>
     </row>
     <row r="33">
       <c r="A33" s="8" t="inlineStr">
@@ -1398,12 +1398,12 @@
           <t>optional</t>
         </is>
       </c>
-      <c r="E33" s="8" t="inlineStr">
+      <c r="E33" s="8" t="n"/>
+      <c r="F33" s="8" t="inlineStr">
         <is>
           <t>hasPositiveElectrode-hasMeasuredProperty-type|RatedCapacity-rev|hasOutput-type|Measurement-hasInput-ConstantCurrentCharging-hasInput-ElectricCurrentDensity</t>
         </is>
       </c>
-      <c r="F33" s="8" t="n"/>
     </row>
     <row r="34">
       <c r="A34" s="4" t="inlineStr">
@@ -1424,12 +1424,12 @@
           <t>optional</t>
         </is>
       </c>
-      <c r="E34" s="4" t="inlineStr">
+      <c r="E34" s="4" t="n"/>
+      <c r="F34" s="4" t="inlineStr">
         <is>
           <t>hasPositiveElectrode-hasMeasuredProperty-type|RatedCapacity-rev|hasOutput-type|Measurement-hasInput-ConstantCurrentCharging-hasInput-UpperVoltageLimit</t>
         </is>
       </c>
-      <c r="F34" s="4" t="n"/>
     </row>
     <row r="35">
       <c r="A35" s="8" t="inlineStr">
@@ -1450,12 +1450,12 @@
           <t>optional</t>
         </is>
       </c>
-      <c r="E35" s="8" t="inlineStr">
+      <c r="E35" s="8" t="n"/>
+      <c r="F35" s="8" t="inlineStr">
         <is>
           <t>hasPositiveElectrode-hasMeasuredProperty-type|RatedCapacity-rev|hasOutput-type|Measurement-hasInput-ConstantVoltageCharging-hasInput-UpperVoltageLimit</t>
         </is>
       </c>
-      <c r="F35" s="8" t="n"/>
     </row>
     <row r="36">
       <c r="A36" s="4" t="inlineStr">
@@ -1476,12 +1476,12 @@
           <t>optional</t>
         </is>
       </c>
-      <c r="E36" s="4" t="inlineStr">
+      <c r="E36" s="4" t="n"/>
+      <c r="F36" s="4" t="inlineStr">
         <is>
           <t>hasPositiveElectrode-hasMeasuredProperty-type|RatedCapacity-rev|hasOutput-type|Measurement-hasInput-ConstantVoltageCharging-hasInput-LowerCurrentDensityLimit</t>
         </is>
       </c>
-      <c r="F36" s="4" t="n"/>
     </row>
     <row r="37">
       <c r="A37" s="8" t="inlineStr">
@@ -1502,12 +1502,12 @@
           <t>optional</t>
         </is>
       </c>
-      <c r="E37" s="8" t="inlineStr">
+      <c r="E37" s="8" t="n"/>
+      <c r="F37" s="8" t="inlineStr">
         <is>
           <t>hasPositiveElectrode-hasMeasuredProperty-type|RatedCapacity-rev|hasOutput-type|Measurement-hasInput-ConstantCurrentDischarging-hasInput-UpperVoltageLimit</t>
         </is>
       </c>
-      <c r="F37" s="8" t="n"/>
     </row>
     <row r="38">
       <c r="A38" s="4" t="inlineStr">
@@ -1528,12 +1528,12 @@
           <t>optional</t>
         </is>
       </c>
-      <c r="E38" s="4" t="inlineStr">
+      <c r="E38" s="4" t="n"/>
+      <c r="F38" s="4" t="inlineStr">
         <is>
           <t>hasPositiveElectrode-hasMeasuredProperty-type|RatedCapacity-rev|hasOutput-type|Measurement-hasInput-ConstantCurrentDischarging-hasInput-ElectricCurrentDensity</t>
         </is>
       </c>
-      <c r="F38" s="4" t="n"/>
     </row>
     <row r="39">
       <c r="A39" s="8" t="inlineStr">
@@ -1554,12 +1554,12 @@
           <t>optional</t>
         </is>
       </c>
-      <c r="E39" s="8" t="inlineStr">
+      <c r="E39" s="8" t="n"/>
+      <c r="F39" s="8" t="inlineStr">
         <is>
           <t>hasPositiveElectrode-hasMeasuredProperty-type|RatedCapacity-rev|hasOutput-type|Measurement-hasInput-ConstantCurrentDischarging-hasInput-LowerVoltageLimit</t>
         </is>
       </c>
-      <c r="F39" s="8" t="n"/>
     </row>
     <row r="40">
       <c r="A40" s="4" t="inlineStr">
@@ -1580,12 +1580,12 @@
           <t>optional</t>
         </is>
       </c>
-      <c r="E40" s="4" t="inlineStr">
+      <c r="E40" s="4" t="n"/>
+      <c r="F40" s="4" t="inlineStr">
         <is>
           <t>hasPositiveElectrode-hasMeasuredProperty-type|RatedCapacity-rev|hasOutput-type|Measurement-hasInput-ConstantVoltageCharging-hasInput-LowerVoltageLimit</t>
         </is>
       </c>
-      <c r="F40" s="4" t="n"/>
     </row>
     <row r="41">
       <c r="A41" s="8" t="inlineStr">
@@ -1606,12 +1606,12 @@
           <t>optional</t>
         </is>
       </c>
-      <c r="E41" s="8" t="inlineStr">
+      <c r="E41" s="8" t="n"/>
+      <c r="F41" s="8" t="inlineStr">
         <is>
           <t>hasPositiveElectrode-hasMeasuredProperty-type|RatedCapacity</t>
         </is>
       </c>
-      <c r="F41" s="8" t="n"/>
     </row>
     <row r="42">
       <c r="A42" s="4" t="inlineStr">
@@ -1632,12 +1632,12 @@
           <t>optional</t>
         </is>
       </c>
-      <c r="E42" s="4" t="inlineStr">
+      <c r="E42" s="4" t="n"/>
+      <c r="F42" s="4" t="inlineStr">
         <is>
           <t>hasPositiveElectrode-hasMeasuredProperty-type|RatedCapacity</t>
         </is>
       </c>
-      <c r="F42" s="4" t="n"/>
     </row>
     <row r="43">
       <c r="A43" s="9" t="inlineStr">
@@ -1672,12 +1672,12 @@
           <t>optional</t>
         </is>
       </c>
-      <c r="E44" s="4" t="inlineStr">
+      <c r="E44" s="4" t="n"/>
+      <c r="F44" s="4" t="inlineStr">
         <is>
           <t>hasPositiveElectrode-schema:manufacturer</t>
         </is>
       </c>
-      <c r="F44" s="4" t="n"/>
     </row>
     <row r="45">
       <c r="A45" s="8" t="inlineStr">
@@ -1698,12 +1698,12 @@
           <t>optional</t>
         </is>
       </c>
-      <c r="E45" s="8" t="inlineStr">
+      <c r="E45" s="8" t="n"/>
+      <c r="F45" s="8" t="inlineStr">
         <is>
           <t>hasPositiveElectrode-schema:productID</t>
         </is>
       </c>
-      <c r="F45" s="8" t="n"/>
     </row>
     <row r="46">
       <c r="A46" s="4" t="inlineStr">
@@ -1722,12 +1722,12 @@
           <t>optional</t>
         </is>
       </c>
-      <c r="E46" s="4" t="inlineStr">
+      <c r="E46" s="4" t="n"/>
+      <c r="F46" s="4" t="inlineStr">
         <is>
           <t>hasPositiveElectrode-hasCurrentCollector-schema:manufacturer</t>
         </is>
       </c>
-      <c r="F46" s="4" t="n"/>
     </row>
     <row r="47">
       <c r="A47" s="8" t="inlineStr">
@@ -1746,12 +1746,12 @@
           <t>optional</t>
         </is>
       </c>
-      <c r="E47" s="8" t="inlineStr">
+      <c r="E47" s="8" t="n"/>
+      <c r="F47" s="8" t="inlineStr">
         <is>
           <t>hasPositiveElectrode-hasCurrentCollector-schema:productID</t>
         </is>
       </c>
-      <c r="F47" s="8" t="n"/>
     </row>
     <row r="48">
       <c r="A48" s="4" t="inlineStr">
@@ -1770,12 +1770,12 @@
           <t>optional</t>
         </is>
       </c>
-      <c r="E48" s="4" t="inlineStr">
+      <c r="E48" s="4" t="n"/>
+      <c r="F48" s="4" t="inlineStr">
         <is>
           <t>hasPositiveElectrode-hasCoating-type|ElectrodeCoating-hasActiveMaterial-schema:manufacturer</t>
         </is>
       </c>
-      <c r="F48" s="4" t="n"/>
     </row>
     <row r="49">
       <c r="A49" s="8" t="inlineStr">
@@ -1794,12 +1794,12 @@
           <t>optional</t>
         </is>
       </c>
-      <c r="E49" s="8" t="inlineStr">
+      <c r="E49" s="8" t="n"/>
+      <c r="F49" s="8" t="inlineStr">
         <is>
           <t>hasPositiveElectrode-hasCoating-type|ElectrodeCoating-hasActiveMaterial-schema:productID</t>
         </is>
       </c>
-      <c r="F49" s="8" t="n"/>
     </row>
     <row r="50">
       <c r="A50" s="4" t="inlineStr">
@@ -1818,12 +1818,12 @@
           <t>optional</t>
         </is>
       </c>
-      <c r="E50" s="4" t="inlineStr">
+      <c r="E50" s="4" t="n"/>
+      <c r="F50" s="4" t="inlineStr">
         <is>
           <t>hasPositiveElectrode-hasCoating-type|ElectrodeCoating-hasBinder-schema:manufacturer</t>
         </is>
       </c>
-      <c r="F50" s="4" t="n"/>
     </row>
     <row r="51">
       <c r="A51" s="8" t="inlineStr">
@@ -1842,12 +1842,12 @@
           <t>optional</t>
         </is>
       </c>
-      <c r="E51" s="8" t="inlineStr">
+      <c r="E51" s="8" t="n"/>
+      <c r="F51" s="8" t="inlineStr">
         <is>
           <t>hasPositiveElectrode-hasCoating-type|ElectrodeCoating-hasBinder-schema:productID</t>
         </is>
       </c>
-      <c r="F51" s="8" t="n"/>
     </row>
     <row r="52">
       <c r="A52" s="4" t="inlineStr">
@@ -1866,12 +1866,12 @@
           <t>optional</t>
         </is>
       </c>
-      <c r="E52" s="4" t="inlineStr">
+      <c r="E52" s="4" t="n"/>
+      <c r="F52" s="4" t="inlineStr">
         <is>
           <t>hasPositiveElectrode-hasCoating-type|ElectrodeCoating-hasConductiveAdditive-schema:manufacturer</t>
         </is>
       </c>
-      <c r="F52" s="4" t="n"/>
     </row>
     <row r="53">
       <c r="A53" s="8" t="inlineStr">
@@ -1890,12 +1890,12 @@
           <t>optional</t>
         </is>
       </c>
-      <c r="E53" s="8" t="inlineStr">
+      <c r="E53" s="8" t="n"/>
+      <c r="F53" s="8" t="inlineStr">
         <is>
           <t>hasPositiveElectrode-hasCoating-type|ElectrodeCoating-hasConductiveAdditive-schema:productID</t>
         </is>
       </c>
-      <c r="F53" s="8" t="n"/>
     </row>
     <row r="54">
       <c r="A54" s="10" t="inlineStr">
@@ -1930,12 +1930,12 @@
           <t>required</t>
         </is>
       </c>
-      <c r="E55" s="4" t="inlineStr">
+      <c r="E55" s="4" t="n"/>
+      <c r="F55" s="4" t="inlineStr">
         <is>
           <t>hasNegativeElectrode-hasCurrentCollector</t>
         </is>
       </c>
-      <c r="F55" s="4" t="n"/>
     </row>
     <row r="56">
       <c r="A56" s="12" t="inlineStr">
@@ -1956,12 +1956,12 @@
           <t>recommended</t>
         </is>
       </c>
-      <c r="E56" s="12" t="inlineStr">
+      <c r="E56" s="12" t="n"/>
+      <c r="F56" s="12" t="inlineStr">
         <is>
           <t>hasNegativeElectrode-hasCurrentCollector-hasMeasuredProperty-Thickness</t>
         </is>
       </c>
-      <c r="F56" s="12" t="n"/>
     </row>
     <row r="57">
       <c r="A57" s="4" t="inlineStr">
@@ -1984,12 +1984,12 @@
           <t>required</t>
         </is>
       </c>
-      <c r="E57" s="4" t="inlineStr">
+      <c r="E57" s="4" t="n"/>
+      <c r="F57" s="4" t="inlineStr">
         <is>
           <t>hasNegativeElectrode-hasCoating-type|ElectrodeCoating-hasActiveMaterial</t>
         </is>
       </c>
-      <c r="F57" s="4" t="n"/>
     </row>
     <row r="58">
       <c r="A58" s="12" t="inlineStr">
@@ -2010,12 +2010,12 @@
           <t>required</t>
         </is>
       </c>
-      <c r="E58" s="12" t="inlineStr">
+      <c r="E58" s="12" t="n"/>
+      <c r="F58" s="12" t="inlineStr">
         <is>
           <t>hasNegativeElectrode-hasCoating-type|ElectrodeCoating-hasActiveMaterial-hasMeasuredProperty-MassFraction</t>
         </is>
       </c>
-      <c r="F58" s="12" t="n"/>
     </row>
     <row r="59">
       <c r="A59" s="4" t="inlineStr">
@@ -2038,12 +2038,12 @@
           <t>required</t>
         </is>
       </c>
-      <c r="E59" s="4" t="inlineStr">
+      <c r="E59" s="4" t="n"/>
+      <c r="F59" s="4" t="inlineStr">
         <is>
           <t>hasNegativeElectrode-hasCoating-type|ElectrodeCoating-hasBinder</t>
         </is>
       </c>
-      <c r="F59" s="4" t="n"/>
     </row>
     <row r="60">
       <c r="A60" s="12" t="inlineStr">
@@ -2064,12 +2064,12 @@
           <t>required</t>
         </is>
       </c>
-      <c r="E60" s="12" t="inlineStr">
+      <c r="E60" s="12" t="n"/>
+      <c r="F60" s="12" t="inlineStr">
         <is>
           <t>hasNegativeElectrode-hasCoating-type|ElectrodeCoating-hasBinder-hasMeasuredProperty-MassFraction</t>
         </is>
       </c>
-      <c r="F60" s="12" t="n"/>
     </row>
     <row r="61">
       <c r="A61" s="4" t="inlineStr">
@@ -2092,12 +2092,12 @@
           <t>required</t>
         </is>
       </c>
-      <c r="E61" s="4" t="inlineStr">
+      <c r="E61" s="4" t="n"/>
+      <c r="F61" s="4" t="inlineStr">
         <is>
           <t>hasNegativeElectrode-hasCoating-type|ElectrodeCoating-hasConductiveAdditive</t>
         </is>
       </c>
-      <c r="F61" s="4" t="n"/>
     </row>
     <row r="62">
       <c r="A62" s="12" t="inlineStr">
@@ -2118,12 +2118,12 @@
           <t>required</t>
         </is>
       </c>
-      <c r="E62" s="12" t="inlineStr">
+      <c r="E62" s="12" t="n"/>
+      <c r="F62" s="12" t="inlineStr">
         <is>
           <t>hasNegativeElectrode-hasCoating-type|ElectrodeCoating-hasConductiveAdditive-hasMeasuredProperty-MassFraction</t>
         </is>
       </c>
-      <c r="F62" s="12" t="n"/>
     </row>
     <row r="63">
       <c r="A63" s="4" t="inlineStr">
@@ -2144,12 +2144,12 @@
           <t>required</t>
         </is>
       </c>
-      <c r="E63" s="4" t="inlineStr">
+      <c r="E63" s="4" t="n"/>
+      <c r="F63" s="4" t="inlineStr">
         <is>
           <t>hasNegativeElectrode-hasCoating-type|ElectrodeCoating-hasActiveMaterial-hasMeasuredProperty-MassLoading</t>
         </is>
       </c>
-      <c r="F63" s="4" t="n"/>
     </row>
     <row r="64">
       <c r="A64" s="12" t="inlineStr">
@@ -2170,12 +2170,12 @@
           <t>recommended</t>
         </is>
       </c>
-      <c r="E64" s="12" t="inlineStr">
+      <c r="E64" s="12" t="n"/>
+      <c r="F64" s="12" t="inlineStr">
         <is>
           <t>hasNegativeElectrode-hasCoating-type|ElectrodeCoating-hasMeasuredProperty-CalenderedCoatingThickness</t>
         </is>
       </c>
-      <c r="F64" s="12" t="n"/>
     </row>
     <row r="65">
       <c r="A65" s="13" t="inlineStr">
@@ -2208,12 +2208,12 @@
           <t>optional</t>
         </is>
       </c>
-      <c r="E66" s="4" t="inlineStr">
+      <c r="E66" s="4" t="n"/>
+      <c r="F66" s="4" t="inlineStr">
         <is>
           <t>hasNegativeElectrode-hasCoating-type|ElectrodeCoating-hasMeasuredProperty-Porosity</t>
         </is>
       </c>
-      <c r="F66" s="4" t="n"/>
     </row>
     <row r="67">
       <c r="A67" s="12" t="inlineStr">
@@ -2234,12 +2234,12 @@
           <t>optional</t>
         </is>
       </c>
-      <c r="E67" s="12" t="inlineStr">
+      <c r="E67" s="12" t="n"/>
+      <c r="F67" s="12" t="inlineStr">
         <is>
           <t>hasNegativeElectrode-hasCoating-type|ElectrodeCoating-hasMeasuredProperty-Tortuosity</t>
         </is>
       </c>
-      <c r="F67" s="12" t="n"/>
     </row>
     <row r="68">
       <c r="A68" s="4" t="inlineStr">
@@ -2260,12 +2260,12 @@
           <t>optional</t>
         </is>
       </c>
-      <c r="E68" s="4" t="inlineStr">
+      <c r="E68" s="4" t="n"/>
+      <c r="F68" s="4" t="inlineStr">
         <is>
           <t>hasNegativeElectrode-hasCoating-type|ElectrodeCoating-hasActiveMaterial-hasMeasuredProperty-D50ParticleSize</t>
         </is>
       </c>
-      <c r="F68" s="4" t="n"/>
     </row>
     <row r="69">
       <c r="A69" s="13" t="inlineStr">
@@ -2300,12 +2300,12 @@
           <t>optional</t>
         </is>
       </c>
-      <c r="E70" s="4" t="inlineStr">
+      <c r="E70" s="4" t="n"/>
+      <c r="F70" s="4" t="inlineStr">
         <is>
           <t>hasNegativeElectrode-hasMeasuredProperty-type|RatedCapacity-rev|hasOutput-type|Measurement-hasInput-ElectrochemicalHalfCell-rdfs:comment</t>
         </is>
       </c>
-      <c r="F70" s="4" t="n"/>
     </row>
     <row r="71">
       <c r="A71" s="12" t="inlineStr">
@@ -2328,12 +2328,12 @@
           <t>optional</t>
         </is>
       </c>
-      <c r="E71" s="12" t="inlineStr">
+      <c r="E71" s="12" t="n"/>
+      <c r="F71" s="12" t="inlineStr">
         <is>
           <t>hasNegativeElectrode-hasMeasuredProperty-type|RatedCapacity-rev|hasOutput-type|Measurement-hasInput-ElectrochemicalHalfCell-hasReferenceElectrode</t>
         </is>
       </c>
-      <c r="F71" s="12" t="n"/>
     </row>
     <row r="72">
       <c r="A72" s="4" t="inlineStr">
@@ -2354,12 +2354,12 @@
           <t>optional</t>
         </is>
       </c>
-      <c r="E72" s="4" t="inlineStr">
+      <c r="E72" s="4" t="n"/>
+      <c r="F72" s="4" t="inlineStr">
         <is>
           <t>hasNegativeElectrode-hasMeasuredProperty-type|RatedCapacity-rev|hasOutput-type|Measurement-hasInput-ConstantCurrentCharging-hasInput-UpperVoltageLimit</t>
         </is>
       </c>
-      <c r="F72" s="4" t="n"/>
     </row>
     <row r="73">
       <c r="A73" s="12" t="inlineStr">
@@ -2380,12 +2380,12 @@
           <t>optional</t>
         </is>
       </c>
-      <c r="E73" s="12" t="inlineStr">
+      <c r="E73" s="12" t="n"/>
+      <c r="F73" s="12" t="inlineStr">
         <is>
           <t>hasNegativeElectrode-hasMeasuredProperty-type|RatedCapacity-rev|hasOutput-type|Measurement-hasInput-ConstantCurrentCharging-hasInput-ElectricCurrentDensity</t>
         </is>
       </c>
-      <c r="F73" s="12" t="n"/>
     </row>
     <row r="74">
       <c r="A74" s="4" t="inlineStr">
@@ -2406,12 +2406,12 @@
           <t>optional</t>
         </is>
       </c>
-      <c r="E74" s="4" t="inlineStr">
+      <c r="E74" s="4" t="n"/>
+      <c r="F74" s="4" t="inlineStr">
         <is>
           <t>hasNegativeElectrode-hasMeasuredProperty-type|RatedCapacity-rev|hasOutput-type|Measurement-hasInput-ConstantCurrentCharging-hasInput-LowerVoltageLimit</t>
         </is>
       </c>
-      <c r="F74" s="4" t="n"/>
     </row>
     <row r="75">
       <c r="A75" s="12" t="inlineStr">
@@ -2432,12 +2432,12 @@
           <t>optional</t>
         </is>
       </c>
-      <c r="E75" s="12" t="inlineStr">
+      <c r="E75" s="12" t="n"/>
+      <c r="F75" s="12" t="inlineStr">
         <is>
           <t>hasNegativeElectrode-hasMeasuredProperty-type|RatedCapacity-rev|hasOutput-type|Measurement-hasInput-ConstantVoltageCharging-hasInput-LowerVoltageLimit</t>
         </is>
       </c>
-      <c r="F75" s="12" t="n"/>
     </row>
     <row r="76">
       <c r="A76" s="4" t="inlineStr">
@@ -2458,12 +2458,12 @@
           <t>optional</t>
         </is>
       </c>
-      <c r="E76" s="4" t="inlineStr">
+      <c r="E76" s="4" t="n"/>
+      <c r="F76" s="4" t="inlineStr">
         <is>
           <t>hasNegativeElectrode-hasMeasuredProperty-type|RatedCapacity-rev|hasOutput-type|Measurement-hasInput-ConstantVoltageCharging-hasInput-LowerCurrentDensityLimit</t>
         </is>
       </c>
-      <c r="F76" s="4" t="n"/>
     </row>
     <row r="77">
       <c r="A77" s="12" t="inlineStr">
@@ -2484,12 +2484,12 @@
           <t>optional</t>
         </is>
       </c>
-      <c r="E77" s="12" t="inlineStr">
+      <c r="E77" s="12" t="n"/>
+      <c r="F77" s="12" t="inlineStr">
         <is>
           <t>hasNegativeElectrode-hasMeasuredProperty-type|RatedCapacity-rev|hasOutput-type|Measurement-hasInput-ConstantCurrentDischarging-hasInput-LowerVoltageLimit</t>
         </is>
       </c>
-      <c r="F77" s="12" t="n"/>
     </row>
     <row r="78">
       <c r="A78" s="4" t="inlineStr">
@@ -2510,12 +2510,12 @@
           <t>optional</t>
         </is>
       </c>
-      <c r="E78" s="4" t="inlineStr">
+      <c r="E78" s="4" t="n"/>
+      <c r="F78" s="4" t="inlineStr">
         <is>
           <t>hasNegativeElectrode-hasMeasuredProperty-type|RatedCapacity-rev|hasOutput-type|Measurement-hasInput-ConstantCurrentDischarging-hasInput-ElectricCurrentDensity</t>
         </is>
       </c>
-      <c r="F78" s="4" t="n"/>
     </row>
     <row r="79">
       <c r="A79" s="12" t="inlineStr">
@@ -2536,12 +2536,12 @@
           <t>optional</t>
         </is>
       </c>
-      <c r="E79" s="12" t="inlineStr">
+      <c r="E79" s="12" t="n"/>
+      <c r="F79" s="12" t="inlineStr">
         <is>
           <t>hasNegativeElectrode-hasMeasuredProperty-type|RatedCapacity-rev|hasOutput-type|Measurement-hasInput-ConstantCurrentDischarging-hasInput-UpperVoltageLimit</t>
         </is>
       </c>
-      <c r="F79" s="12" t="n"/>
     </row>
     <row r="80">
       <c r="A80" s="4" t="inlineStr">
@@ -2562,12 +2562,12 @@
           <t>optional</t>
         </is>
       </c>
-      <c r="E80" s="4" t="inlineStr">
+      <c r="E80" s="4" t="n"/>
+      <c r="F80" s="4" t="inlineStr">
         <is>
           <t>hasNegativeElectrode-hasMeasuredProperty-type|RatedCapacity-rev|hasOutput-type|Measurement-hasInput-ConstantVoltageCharging-hasInput-UpperVoltageLimit</t>
         </is>
       </c>
-      <c r="F80" s="4" t="n"/>
     </row>
     <row r="81">
       <c r="A81" s="12" t="inlineStr">
@@ -2588,12 +2588,12 @@
           <t>optional</t>
         </is>
       </c>
-      <c r="E81" s="12" t="inlineStr">
+      <c r="E81" s="12" t="n"/>
+      <c r="F81" s="12" t="inlineStr">
         <is>
           <t>hasNegativeElectrode-hasMeasuredProperty-type|RatedCapacity</t>
         </is>
       </c>
-      <c r="F81" s="12" t="n"/>
     </row>
     <row r="82">
       <c r="A82" s="4" t="inlineStr">
@@ -2614,12 +2614,12 @@
           <t>optional</t>
         </is>
       </c>
-      <c r="E82" s="4" t="inlineStr">
+      <c r="E82" s="4" t="n"/>
+      <c r="F82" s="4" t="inlineStr">
         <is>
           <t>hasNegativeElectrode-hasMeasuredProperty-type|RatedCapacity</t>
         </is>
       </c>
-      <c r="F82" s="4" t="n"/>
     </row>
     <row r="83">
       <c r="A83" s="13" t="inlineStr">
@@ -2654,12 +2654,12 @@
           <t>optional</t>
         </is>
       </c>
-      <c r="E84" s="4" t="inlineStr">
+      <c r="E84" s="4" t="n"/>
+      <c r="F84" s="4" t="inlineStr">
         <is>
           <t>hasNegativeElectrode-schema:manufacturer</t>
         </is>
       </c>
-      <c r="F84" s="4" t="n"/>
     </row>
     <row r="85">
       <c r="A85" s="12" t="inlineStr">
@@ -2682,12 +2682,12 @@
           <t>optional</t>
         </is>
       </c>
-      <c r="E85" s="12" t="inlineStr">
+      <c r="E85" s="12" t="n"/>
+      <c r="F85" s="12" t="inlineStr">
         <is>
           <t>hasNegativeElectrode-schema:productID</t>
         </is>
       </c>
-      <c r="F85" s="12" t="n"/>
     </row>
     <row r="86">
       <c r="A86" s="4" t="inlineStr">
@@ -2706,12 +2706,12 @@
           <t>optional</t>
         </is>
       </c>
-      <c r="E86" s="4" t="inlineStr">
+      <c r="E86" s="4" t="n"/>
+      <c r="F86" s="4" t="inlineStr">
         <is>
           <t>hasNegativeElectrode-hasCurrentCollector-schema:manufacturer</t>
         </is>
       </c>
-      <c r="F86" s="4" t="n"/>
     </row>
     <row r="87">
       <c r="A87" s="12" t="inlineStr">
@@ -2730,12 +2730,12 @@
           <t>optional</t>
         </is>
       </c>
-      <c r="E87" s="12" t="inlineStr">
+      <c r="E87" s="12" t="n"/>
+      <c r="F87" s="12" t="inlineStr">
         <is>
           <t>hasNegativeElectrode-hasCurrentCollector-schema:productID</t>
         </is>
       </c>
-      <c r="F87" s="12" t="n"/>
     </row>
     <row r="88">
       <c r="A88" s="4" t="inlineStr">
@@ -2754,12 +2754,12 @@
           <t>optional</t>
         </is>
       </c>
-      <c r="E88" s="4" t="inlineStr">
+      <c r="E88" s="4" t="n"/>
+      <c r="F88" s="4" t="inlineStr">
         <is>
           <t>hasNegativeElectrode-hasCoating-type|ElectrodeCoating-hasActiveMaterial-schema:manufacturer</t>
         </is>
       </c>
-      <c r="F88" s="4" t="n"/>
     </row>
     <row r="89">
       <c r="A89" s="12" t="inlineStr">
@@ -2778,12 +2778,12 @@
           <t>optional</t>
         </is>
       </c>
-      <c r="E89" s="12" t="inlineStr">
+      <c r="E89" s="12" t="n"/>
+      <c r="F89" s="12" t="inlineStr">
         <is>
           <t>hasNegativeElectrode-hasCoating-type|ElectrodeCoating-hasActiveMaterial-schema:productID</t>
         </is>
       </c>
-      <c r="F89" s="12" t="n"/>
     </row>
     <row r="90">
       <c r="A90" s="4" t="inlineStr">
@@ -2802,12 +2802,12 @@
           <t>optional</t>
         </is>
       </c>
-      <c r="E90" s="4" t="inlineStr">
+      <c r="E90" s="4" t="n"/>
+      <c r="F90" s="4" t="inlineStr">
         <is>
           <t>hasNegativeElectrode-hasCoating-type|ElectrodeCoating-hasBinder-schema:manufacturer</t>
         </is>
       </c>
-      <c r="F90" s="4" t="n"/>
     </row>
     <row r="91">
       <c r="A91" s="12" t="inlineStr">
@@ -2826,12 +2826,12 @@
           <t>optional</t>
         </is>
       </c>
-      <c r="E91" s="12" t="inlineStr">
+      <c r="E91" s="12" t="n"/>
+      <c r="F91" s="12" t="inlineStr">
         <is>
           <t>hasNegativeElectrode-hasCoating-type|ElectrodeCoating-hasBinder-schema:productID</t>
         </is>
       </c>
-      <c r="F91" s="12" t="n"/>
     </row>
     <row r="92">
       <c r="A92" s="4" t="inlineStr">
@@ -2850,12 +2850,12 @@
           <t>optional</t>
         </is>
       </c>
-      <c r="E92" s="4" t="inlineStr">
+      <c r="E92" s="4" t="n"/>
+      <c r="F92" s="4" t="inlineStr">
         <is>
           <t>hasNegativeElectrode-hasCoating-type|ElectrodeCoating-hasConductiveAdditive-schema:manufacturer</t>
         </is>
       </c>
-      <c r="F92" s="4" t="n"/>
     </row>
     <row r="93">
       <c r="A93" s="12" t="inlineStr">
@@ -2874,12 +2874,12 @@
           <t>optional</t>
         </is>
       </c>
-      <c r="E93" s="12" t="inlineStr">
+      <c r="E93" s="12" t="n"/>
+      <c r="F93" s="12" t="inlineStr">
         <is>
           <t>hasNegativeElectrode-hasCoating-type|ElectrodeCoating-hasConductiveAdditive-schema:productID</t>
         </is>
       </c>
-      <c r="F93" s="12" t="n"/>
     </row>
     <row r="94">
       <c r="A94" s="14" t="inlineStr">
@@ -2914,12 +2914,12 @@
           <t>required</t>
         </is>
       </c>
-      <c r="E95" s="4" t="inlineStr">
+      <c r="E95" s="4" t="n"/>
+      <c r="F95" s="4" t="inlineStr">
         <is>
           <t>hasElectrolyte-hasSolvent-hasConstituentA</t>
         </is>
       </c>
-      <c r="F95" s="4" t="n"/>
     </row>
     <row r="96">
       <c r="A96" s="16" t="inlineStr">
@@ -2940,12 +2940,12 @@
           <t>required</t>
         </is>
       </c>
-      <c r="E96" s="16" t="inlineStr">
+      <c r="E96" s="16" t="n"/>
+      <c r="F96" s="16" t="inlineStr">
         <is>
           <t>hasElectrolyte-hasSolvent-hasConstituentA-hasMeasuredProperty-VolumeFraction</t>
         </is>
       </c>
-      <c r="F96" s="16" t="n"/>
     </row>
     <row r="97">
       <c r="A97" s="4" t="inlineStr">
@@ -2968,12 +2968,12 @@
           <t>recommended</t>
         </is>
       </c>
-      <c r="E97" s="4" t="inlineStr">
+      <c r="E97" s="4" t="n"/>
+      <c r="F97" s="4" t="inlineStr">
         <is>
           <t>hasElectrolyte-hasSolvent-hasConstituentB</t>
         </is>
       </c>
-      <c r="F97" s="4" t="n"/>
     </row>
     <row r="98">
       <c r="A98" s="16" t="inlineStr">
@@ -2994,12 +2994,12 @@
           <t>recommended</t>
         </is>
       </c>
-      <c r="E98" s="16" t="inlineStr">
+      <c r="E98" s="16" t="n"/>
+      <c r="F98" s="16" t="inlineStr">
         <is>
           <t>hasElectrolyte-hasSolvent-hasConstituentB-hasMeasuredProperty-VolumeFraction</t>
         </is>
       </c>
-      <c r="F98" s="16" t="n"/>
     </row>
     <row r="99">
       <c r="A99" s="4" t="inlineStr">
@@ -3022,12 +3022,12 @@
           <t>required</t>
         </is>
       </c>
-      <c r="E99" s="4" t="inlineStr">
+      <c r="E99" s="4" t="n"/>
+      <c r="F99" s="4" t="inlineStr">
         <is>
           <t>hasElectrolyte-hasSolute-hasConstituentA</t>
         </is>
       </c>
-      <c r="F99" s="4" t="n"/>
     </row>
     <row r="100">
       <c r="A100" s="16" t="inlineStr">
@@ -3048,12 +3048,12 @@
           <t>required</t>
         </is>
       </c>
-      <c r="E100" s="16" t="inlineStr">
+      <c r="E100" s="16" t="n"/>
+      <c r="F100" s="16" t="inlineStr">
         <is>
           <t>hasElectrolyte-hasSolute-hasConstituentA-hasMeasuredProperty-AmountConcentration</t>
         </is>
       </c>
-      <c r="F100" s="16" t="n"/>
     </row>
     <row r="101">
       <c r="A101" s="4" t="inlineStr">
@@ -3076,12 +3076,12 @@
           <t>optional</t>
         </is>
       </c>
-      <c r="E101" s="4" t="inlineStr">
+      <c r="E101" s="4" t="n"/>
+      <c r="F101" s="4" t="inlineStr">
         <is>
           <t>hasElectrolyte-hasSolute-hasConstituentB</t>
         </is>
       </c>
-      <c r="F101" s="4" t="n"/>
     </row>
     <row r="102">
       <c r="A102" s="16" t="inlineStr">
@@ -3102,12 +3102,12 @@
           <t>optional</t>
         </is>
       </c>
-      <c r="E102" s="16" t="inlineStr">
+      <c r="E102" s="16" t="n"/>
+      <c r="F102" s="16" t="inlineStr">
         <is>
           <t>hasElectrolyte-hasSolute-hasConstituentB-hasMeasuredProperty-AmountConcentration</t>
         </is>
       </c>
-      <c r="F102" s="16" t="n"/>
     </row>
     <row r="103">
       <c r="A103" s="4" t="inlineStr">
@@ -3130,12 +3130,12 @@
           <t>optional</t>
         </is>
       </c>
-      <c r="E103" s="4" t="inlineStr">
+      <c r="E103" s="4" t="n"/>
+      <c r="F103" s="4" t="inlineStr">
         <is>
           <t>hasElectrolyte-hasSolute-hasAdditive-hasConstituentA</t>
         </is>
       </c>
-      <c r="F103" s="4" t="n"/>
     </row>
     <row r="104">
       <c r="A104" s="16" t="inlineStr">
@@ -3156,12 +3156,12 @@
           <t>optional</t>
         </is>
       </c>
-      <c r="E104" s="16" t="inlineStr">
+      <c r="E104" s="16" t="n"/>
+      <c r="F104" s="16" t="inlineStr">
         <is>
           <t>hasElectrolyte-hasSolute-hasAdditive-hasConstituentA-hasMeasuredProperty-AmountConcentration</t>
         </is>
       </c>
-      <c r="F104" s="16" t="n"/>
     </row>
     <row r="105">
       <c r="A105" s="4" t="inlineStr">
@@ -3184,12 +3184,12 @@
           <t>optional</t>
         </is>
       </c>
-      <c r="E105" s="4" t="inlineStr">
+      <c r="E105" s="4" t="n"/>
+      <c r="F105" s="4" t="inlineStr">
         <is>
           <t>hasElectrolyte-hasSolute-hasAdditive-hasConstituentB</t>
         </is>
       </c>
-      <c r="F105" s="4" t="n"/>
     </row>
     <row r="106">
       <c r="A106" s="16" t="inlineStr">
@@ -3210,12 +3210,12 @@
           <t>optional</t>
         </is>
       </c>
-      <c r="E106" s="16" t="inlineStr">
+      <c r="E106" s="16" t="n"/>
+      <c r="F106" s="16" t="inlineStr">
         <is>
           <t>hasElectrolyte-hasSolute-hasAdditive-hasConstituentB-hasMeasuredProperty-AmountConcentration</t>
         </is>
       </c>
-      <c r="F106" s="16" t="n"/>
     </row>
     <row r="107">
       <c r="A107" s="17" t="inlineStr">
@@ -3248,12 +3248,12 @@
           <t>optional</t>
         </is>
       </c>
-      <c r="E108" s="4" t="inlineStr">
+      <c r="E108" s="4" t="n"/>
+      <c r="F108" s="4" t="inlineStr">
         <is>
           <t>hasElectrolyte-hasMeasuredProperty-ElectrolyticConductivity</t>
         </is>
       </c>
-      <c r="F108" s="4" t="n"/>
     </row>
     <row r="109">
       <c r="A109" s="16" t="inlineStr">
@@ -3274,12 +3274,12 @@
           <t>optional</t>
         </is>
       </c>
-      <c r="E109" s="16" t="inlineStr">
+      <c r="E109" s="16" t="n"/>
+      <c r="F109" s="16" t="inlineStr">
         <is>
           <t>hasElectrolyte-hasMeasuredProperty-DynamicViscosity</t>
         </is>
       </c>
-      <c r="F109" s="16" t="n"/>
     </row>
     <row r="110">
       <c r="A110" s="4" t="inlineStr">
@@ -3300,12 +3300,12 @@
           <t>optional</t>
         </is>
       </c>
-      <c r="E110" s="4" t="inlineStr">
+      <c r="E110" s="4" t="n"/>
+      <c r="F110" s="4" t="inlineStr">
         <is>
           <t>hasElectrolyte-hasMeasuredProperty-Density</t>
         </is>
       </c>
-      <c r="F110" s="4" t="n"/>
     </row>
     <row r="111">
       <c r="A111" s="16" t="inlineStr">
@@ -3326,12 +3326,12 @@
           <t>optional</t>
         </is>
       </c>
-      <c r="E111" s="16" t="inlineStr">
+      <c r="E111" s="16" t="n"/>
+      <c r="F111" s="16" t="inlineStr">
         <is>
           <t>hasElectrolyte-hasMeasuredProperty-CelsiusTemperature</t>
         </is>
       </c>
-      <c r="F111" s="16" t="n"/>
     </row>
     <row r="112">
       <c r="A112" s="17" t="inlineStr">
@@ -3366,12 +3366,12 @@
           <t>optional</t>
         </is>
       </c>
-      <c r="E113" s="4" t="inlineStr">
+      <c r="E113" s="4" t="n"/>
+      <c r="F113" s="4" t="inlineStr">
         <is>
           <t>hasElectrolyte-schema:manufacturer</t>
         </is>
       </c>
-      <c r="F113" s="4" t="n"/>
     </row>
     <row r="114">
       <c r="A114" s="16" t="inlineStr">
@@ -3390,12 +3390,12 @@
           <t>optional</t>
         </is>
       </c>
-      <c r="E114" s="16" t="inlineStr">
+      <c r="E114" s="16" t="n"/>
+      <c r="F114" s="16" t="inlineStr">
         <is>
           <t>hasElectrolyte-schema:productID</t>
         </is>
       </c>
-      <c r="F114" s="16" t="n"/>
     </row>
     <row r="115">
       <c r="A115" s="4" t="inlineStr">
@@ -3414,12 +3414,12 @@
           <t>optional</t>
         </is>
       </c>
-      <c r="E115" s="4" t="inlineStr">
+      <c r="E115" s="4" t="n"/>
+      <c r="F115" s="4" t="inlineStr">
         <is>
           <t>hasElectrolyte-hasSolvent-hasConstituentA-schema:manufacturer</t>
         </is>
       </c>
-      <c r="F115" s="4" t="n"/>
     </row>
     <row r="116">
       <c r="A116" s="16" t="inlineStr">
@@ -3438,12 +3438,12 @@
           <t>optional</t>
         </is>
       </c>
-      <c r="E116" s="16" t="inlineStr">
+      <c r="E116" s="16" t="n"/>
+      <c r="F116" s="16" t="inlineStr">
         <is>
           <t>hasElectrolyte-hasSolvent-hasConstituentA-schema:productID</t>
         </is>
       </c>
-      <c r="F116" s="16" t="n"/>
     </row>
     <row r="117">
       <c r="A117" s="4" t="inlineStr">
@@ -3462,12 +3462,12 @@
           <t>optional</t>
         </is>
       </c>
-      <c r="E117" s="4" t="inlineStr">
+      <c r="E117" s="4" t="n"/>
+      <c r="F117" s="4" t="inlineStr">
         <is>
           <t>hasElectrolyte-hasSolvent-hasConstituentB-schema:manufacturer</t>
         </is>
       </c>
-      <c r="F117" s="4" t="n"/>
     </row>
     <row r="118">
       <c r="A118" s="16" t="inlineStr">
@@ -3486,12 +3486,12 @@
           <t>optional</t>
         </is>
       </c>
-      <c r="E118" s="16" t="inlineStr">
+      <c r="E118" s="16" t="n"/>
+      <c r="F118" s="16" t="inlineStr">
         <is>
           <t>hasElectrolyte-hasSolvent-hasConstituentB-schema:productID</t>
         </is>
       </c>
-      <c r="F118" s="16" t="n"/>
     </row>
     <row r="119">
       <c r="A119" s="4" t="inlineStr">
@@ -3510,12 +3510,12 @@
           <t>optional</t>
         </is>
       </c>
-      <c r="E119" s="4" t="inlineStr">
+      <c r="E119" s="4" t="n"/>
+      <c r="F119" s="4" t="inlineStr">
         <is>
           <t>hasElectrolyte-hasSolute-hasConstituentA-schema:manufacturer</t>
         </is>
       </c>
-      <c r="F119" s="4" t="n"/>
     </row>
     <row r="120">
       <c r="A120" s="16" t="inlineStr">
@@ -3534,12 +3534,12 @@
           <t>optional</t>
         </is>
       </c>
-      <c r="E120" s="16" t="inlineStr">
+      <c r="E120" s="16" t="n"/>
+      <c r="F120" s="16" t="inlineStr">
         <is>
           <t>hasElectrolyte-hasSolute-hasConstituentA-schema:productID</t>
         </is>
       </c>
-      <c r="F120" s="16" t="n"/>
     </row>
     <row r="121">
       <c r="A121" s="4" t="inlineStr">
@@ -3558,12 +3558,12 @@
           <t>optional</t>
         </is>
       </c>
-      <c r="E121" s="4" t="inlineStr">
+      <c r="E121" s="4" t="n"/>
+      <c r="F121" s="4" t="inlineStr">
         <is>
           <t>hasElectrolyte-hasSolute-hasConstituentB-schema:manufacturer</t>
         </is>
       </c>
-      <c r="F121" s="4" t="n"/>
     </row>
     <row r="122">
       <c r="A122" s="16" t="inlineStr">
@@ -3582,12 +3582,12 @@
           <t>optional</t>
         </is>
       </c>
-      <c r="E122" s="16" t="inlineStr">
+      <c r="E122" s="16" t="n"/>
+      <c r="F122" s="16" t="inlineStr">
         <is>
           <t>hasElectrolyte-hasSolute-hasConstituentB-schema:productID</t>
         </is>
       </c>
-      <c r="F122" s="16" t="n"/>
     </row>
     <row r="123">
       <c r="A123" s="4" t="inlineStr">
@@ -3606,12 +3606,12 @@
           <t>optional</t>
         </is>
       </c>
-      <c r="E123" s="4" t="inlineStr">
+      <c r="E123" s="4" t="n"/>
+      <c r="F123" s="4" t="inlineStr">
         <is>
           <t>hasElectrolyte-hasSolute-hasAdditive-hasConstituentA-schema:manufacturer</t>
         </is>
       </c>
-      <c r="F123" s="4" t="n"/>
     </row>
     <row r="124">
       <c r="A124" s="16" t="inlineStr">
@@ -3630,12 +3630,12 @@
           <t>optional</t>
         </is>
       </c>
-      <c r="E124" s="16" t="inlineStr">
+      <c r="E124" s="16" t="n"/>
+      <c r="F124" s="16" t="inlineStr">
         <is>
           <t>hasElectrolyte-hasSolute-hasAdditive-hasConstituentA-schema:productID</t>
         </is>
       </c>
-      <c r="F124" s="16" t="n"/>
     </row>
     <row r="125">
       <c r="A125" s="4" t="inlineStr">
@@ -3654,12 +3654,12 @@
           <t>optional</t>
         </is>
       </c>
-      <c r="E125" s="4" t="inlineStr">
+      <c r="E125" s="4" t="n"/>
+      <c r="F125" s="4" t="inlineStr">
         <is>
           <t>hasElectrolyte-hasSolute-hasAdditive-hasConstituentB-schema:manufacturer</t>
         </is>
       </c>
-      <c r="F125" s="4" t="n"/>
     </row>
     <row r="126">
       <c r="A126" s="16" t="inlineStr">
@@ -3678,12 +3678,12 @@
           <t>optional</t>
         </is>
       </c>
-      <c r="E126" s="16" t="inlineStr">
+      <c r="E126" s="16" t="n"/>
+      <c r="F126" s="16" t="inlineStr">
         <is>
           <t>hasElectrolyte-hasSolute-hasAdditive-hasConstituentB-schema:productID</t>
         </is>
       </c>
-      <c r="F126" s="16" t="n"/>
     </row>
     <row r="127">
       <c r="A127" s="2" t="inlineStr">
@@ -3718,12 +3718,12 @@
           <t>required</t>
         </is>
       </c>
-      <c r="E128" s="4" t="inlineStr">
+      <c r="E128" s="4" t="n"/>
+      <c r="F128" s="4" t="inlineStr">
         <is>
           <t>hasSeparator</t>
         </is>
       </c>
-      <c r="F128" s="4" t="n"/>
     </row>
     <row r="129">
       <c r="A129" s="5" t="inlineStr">
@@ -3744,12 +3744,12 @@
           <t>required</t>
         </is>
       </c>
-      <c r="E129" s="5" t="inlineStr">
+      <c r="E129" s="5" t="n"/>
+      <c r="F129" s="5" t="inlineStr">
         <is>
           <t>hasSeparator-hasMeasuredProperty-Thickness</t>
         </is>
       </c>
-      <c r="F129" s="5" t="n"/>
     </row>
     <row r="130">
       <c r="A130" s="18" t="inlineStr">
@@ -3782,12 +3782,12 @@
           <t>recommended</t>
         </is>
       </c>
-      <c r="E131" s="4" t="inlineStr">
+      <c r="E131" s="4" t="n"/>
+      <c r="F131" s="4" t="inlineStr">
         <is>
           <t>hasSeparator-hasMeasuredProperty-Porosity</t>
         </is>
       </c>
-      <c r="F131" s="4" t="n"/>
     </row>
     <row r="132">
       <c r="A132" s="5" t="inlineStr">
@@ -3808,12 +3808,12 @@
           <t>optional</t>
         </is>
       </c>
-      <c r="E132" s="5" t="inlineStr">
+      <c r="E132" s="5" t="n"/>
+      <c r="F132" s="5" t="inlineStr">
         <is>
           <t>hasSeparator-hasMeasuredProperty-Tortuosity</t>
         </is>
       </c>
-      <c r="F132" s="5" t="n"/>
     </row>
     <row r="133">
       <c r="A133" s="18" t="inlineStr">
@@ -3848,12 +3848,12 @@
           <t>optional</t>
         </is>
       </c>
-      <c r="E134" s="4" t="inlineStr">
+      <c r="E134" s="4" t="n"/>
+      <c r="F134" s="4" t="inlineStr">
         <is>
           <t>hasSeparator-schema:manufacturer</t>
         </is>
       </c>
-      <c r="F134" s="4" t="n"/>
     </row>
     <row r="135">
       <c r="A135" s="5" t="inlineStr">
@@ -3874,12 +3874,12 @@
           <t>optional</t>
         </is>
       </c>
-      <c r="E135" s="5" t="inlineStr">
+      <c r="E135" s="5" t="n"/>
+      <c r="F135" s="5" t="inlineStr">
         <is>
           <t>hasSeparator-schema:productID</t>
         </is>
       </c>
-      <c r="F135" s="5" t="n"/>
     </row>
     <row r="136">
       <c r="A136" s="2" t="inlineStr">
@@ -3914,12 +3914,12 @@
           <t>required</t>
         </is>
       </c>
-      <c r="E137" s="4" t="inlineStr">
+      <c r="E137" s="4" t="n"/>
+      <c r="F137" s="4" t="inlineStr">
         <is>
           <t>hasCase</t>
         </is>
       </c>
-      <c r="F137" s="4" t="n"/>
     </row>
     <row r="138">
       <c r="A138" s="5" t="inlineStr">
@@ -3942,12 +3942,12 @@
           <t>required</t>
         </is>
       </c>
-      <c r="E138" s="5" t="inlineStr">
+      <c r="E138" s="5" t="n"/>
+      <c r="F138" s="5" t="inlineStr">
         <is>
           <t>hasCase</t>
         </is>
       </c>
-      <c r="F138" s="5" t="n"/>
     </row>
     <row r="139">
       <c r="A139" s="4" t="inlineStr">
@@ -3970,12 +3970,12 @@
           <t>required</t>
         </is>
       </c>
-      <c r="E139" s="4" t="inlineStr">
+      <c r="E139" s="4" t="n"/>
+      <c r="F139" s="4" t="inlineStr">
         <is>
           <t>hasCase-hasComponentA-type|CellLid-hasCoating</t>
         </is>
       </c>
-      <c r="F139" s="4" t="n"/>
     </row>
     <row r="140">
       <c r="A140" s="5" t="inlineStr">
@@ -3998,12 +3998,12 @@
           <t>required</t>
         </is>
       </c>
-      <c r="E140" s="5" t="inlineStr">
+      <c r="E140" s="5" t="n"/>
+      <c r="F140" s="5" t="inlineStr">
         <is>
           <t>hasCase-hasComponentB-type|CellCan-hasCoating</t>
         </is>
       </c>
-      <c r="F140" s="5" t="n"/>
     </row>
     <row r="141">
       <c r="A141" s="4" t="inlineStr">
@@ -4024,12 +4024,12 @@
           <t>required</t>
         </is>
       </c>
-      <c r="E141" s="4" t="inlineStr">
+      <c r="E141" s="4" t="n"/>
+      <c r="F141" s="4" t="inlineStr">
         <is>
           <t>hasComponentA-type|Spring-hasMeasuredProperty-Diameter</t>
         </is>
       </c>
-      <c r="F141" s="4" t="n"/>
     </row>
     <row r="142">
       <c r="A142" s="5" t="inlineStr">
@@ -4050,12 +4050,12 @@
           <t>required</t>
         </is>
       </c>
-      <c r="E142" s="5" t="inlineStr">
+      <c r="E142" s="5" t="n"/>
+      <c r="F142" s="5" t="inlineStr">
         <is>
           <t>hasComponentA-type|Spring-hasMeasuredProperty-Thickness</t>
         </is>
       </c>
-      <c r="F142" s="5" t="n"/>
     </row>
     <row r="143">
       <c r="A143" s="4" t="inlineStr">
@@ -4076,12 +4076,12 @@
           <t>required</t>
         </is>
       </c>
-      <c r="E143" s="4" t="inlineStr">
+      <c r="E143" s="4" t="n"/>
+      <c r="F143" s="4" t="inlineStr">
         <is>
           <t>hasComponentB-type|Spacer-hasMeasuredProperty-Diameter</t>
         </is>
       </c>
-      <c r="F143" s="4" t="n"/>
     </row>
     <row r="144">
       <c r="A144" s="5" t="inlineStr">
@@ -4102,12 +4102,12 @@
           <t>required</t>
         </is>
       </c>
-      <c r="E144" s="5" t="inlineStr">
+      <c r="E144" s="5" t="n"/>
+      <c r="F144" s="5" t="inlineStr">
         <is>
           <t>hasComponentB-type|Spacer-hasMeasuredProperty-Thickness</t>
         </is>
       </c>
-      <c r="F144" s="5" t="n"/>
     </row>
     <row r="145">
       <c r="A145" s="4" t="inlineStr">
@@ -4128,12 +4128,12 @@
           <t>required</t>
         </is>
       </c>
-      <c r="E145" s="4" t="inlineStr">
+      <c r="E145" s="4" t="n"/>
+      <c r="F145" s="4" t="inlineStr">
         <is>
           <t>hasPositiveElectrode-hasMeasuredProperty-Diameter</t>
         </is>
       </c>
-      <c r="F145" s="4" t="n"/>
     </row>
     <row r="146">
       <c r="A146" s="5" t="inlineStr">
@@ -4154,12 +4154,12 @@
           <t>recommended</t>
         </is>
       </c>
-      <c r="E146" s="5" t="inlineStr">
+      <c r="E146" s="5" t="n"/>
+      <c r="F146" s="5" t="inlineStr">
         <is>
           <t>hasNegativeElectrode-hasMeasuredProperty-Diameter</t>
         </is>
       </c>
-      <c r="F146" s="5" t="n"/>
     </row>
     <row r="147">
       <c r="A147" s="4" t="inlineStr">
@@ -4180,12 +4180,12 @@
           <t>recommended</t>
         </is>
       </c>
-      <c r="E147" s="4" t="inlineStr">
+      <c r="E147" s="4" t="n"/>
+      <c r="F147" s="4" t="inlineStr">
         <is>
           <t>hasSeparator-hasMeasuredProperty-Diameter</t>
         </is>
       </c>
-      <c r="F147" s="4" t="n"/>
     </row>
     <row r="148">
       <c r="A148" s="5" t="inlineStr">
@@ -4206,12 +4206,12 @@
           <t>required</t>
         </is>
       </c>
-      <c r="E148" s="5" t="inlineStr">
+      <c r="E148" s="5" t="n"/>
+      <c r="F148" s="5" t="inlineStr">
         <is>
           <t>hasElectrolyte-hasMeasuredProperty-Volume</t>
         </is>
       </c>
-      <c r="F148" s="5" t="n"/>
     </row>
     <row r="149">
       <c r="A149" s="4" t="inlineStr">
@@ -4234,12 +4234,12 @@
           <t>optional</t>
         </is>
       </c>
-      <c r="E149" s="4" t="inlineStr">
+      <c r="E149" s="4" t="n"/>
+      <c r="F149" s="4" t="inlineStr">
         <is>
           <t>rdfs:comment</t>
         </is>
       </c>
-      <c r="F149" s="4" t="n"/>
     </row>
     <row r="150">
       <c r="A150" s="18" t="inlineStr">
@@ -4274,12 +4274,12 @@
           <t>optional</t>
         </is>
       </c>
-      <c r="E151" s="4" t="inlineStr">
+      <c r="E151" s="4" t="n"/>
+      <c r="F151" s="4" t="inlineStr">
         <is>
           <t>hasCase-schema:manufacturer</t>
         </is>
       </c>
-      <c r="F151" s="4" t="n"/>
     </row>
     <row r="152">
       <c r="A152" s="5" t="inlineStr">
@@ -4302,12 +4302,12 @@
           <t>optional</t>
         </is>
       </c>
-      <c r="E152" s="5" t="inlineStr">
+      <c r="E152" s="5" t="n"/>
+      <c r="F152" s="5" t="inlineStr">
         <is>
           <t>hasCase-schema:productID</t>
         </is>
       </c>
-      <c r="F152" s="5" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Switch ontology link and comment cols (#81)
</commit_message>
<xml_diff>
--- a/test/data/coincell_excel_schema.xlsx
+++ b/test/data/coincell_excel_schema.xlsx
@@ -523,8 +523,8 @@
     <col width="42" customWidth="1" min="2" max="2"/>
     <col width="9" customWidth="1" min="3" max="3"/>
     <col width="14" customWidth="1" min="4" max="4"/>
-    <col width="160" customWidth="1" min="5" max="5"/>
-    <col width="74" customWidth="1" min="6" max="6"/>
+    <col width="74" customWidth="1" min="5" max="5"/>
+    <col width="160" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1" ht="20" customHeight="1">
@@ -550,12 +550,12 @@
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
+          <t>Comment</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
           <t>Ontology link</t>
-        </is>
-      </c>
-      <c r="F1" s="1" t="inlineStr">
-        <is>
-          <t>Comment</t>
         </is>
       </c>
     </row>
@@ -594,12 +594,12 @@
       </c>
       <c r="E3" s="4" t="inlineStr">
         <is>
+          <t>Required, do not change</t>
+        </is>
+      </c>
+      <c r="F3" s="4" t="inlineStr">
+        <is>
           <t>type|</t>
-        </is>
-      </c>
-      <c r="F3" s="4" t="inlineStr">
-        <is>
-          <t>Required, do not change</t>
         </is>
       </c>
     </row>
@@ -626,12 +626,12 @@
       </c>
       <c r="E4" s="5" t="inlineStr">
         <is>
+          <t>Unique ID for cell</t>
+        </is>
+      </c>
+      <c r="F4" s="5" t="inlineStr">
+        <is>
           <t>schema:productID</t>
-        </is>
-      </c>
-      <c r="F4" s="5" t="inlineStr">
-        <is>
-          <t>Unique ID for cell</t>
         </is>
       </c>
     </row>
@@ -658,12 +658,12 @@
       </c>
       <c r="E5" s="4" t="inlineStr">
         <is>
+          <t>Human-friendly name for the cell</t>
+        </is>
+      </c>
+      <c r="F5" s="4" t="inlineStr">
+        <is>
           <t>schema:name</t>
-        </is>
-      </c>
-      <c r="F5" s="4" t="inlineStr">
-        <is>
-          <t>Human-friendly name for the cell</t>
         </is>
       </c>
     </row>
@@ -690,12 +690,12 @@
       </c>
       <c r="E6" s="5" t="inlineStr">
         <is>
+          <t>Assembly date in ISO8601 format (YYYY-MM-DD)</t>
+        </is>
+      </c>
+      <c r="F6" s="5" t="inlineStr">
+        <is>
           <t>schema:dateCreated</t>
-        </is>
-      </c>
-      <c r="F6" s="5" t="inlineStr">
-        <is>
-          <t>Assembly date in ISO8601 format (YYYY-MM-DD)</t>
         </is>
       </c>
     </row>
@@ -722,12 +722,12 @@
       </c>
       <c r="E7" s="4" t="inlineStr">
         <is>
+          <t>Organisation that made the cell, value should be in @classes with ID</t>
+        </is>
+      </c>
+      <c r="F7" s="4" t="inlineStr">
+        <is>
           <t>schema:manufacturer</t>
-        </is>
-      </c>
-      <c r="F7" s="4" t="inlineStr">
-        <is>
-          <t>Organisation that made the cell, value should be in @classes with ID</t>
         </is>
       </c>
     </row>
@@ -754,12 +754,12 @@
       </c>
       <c r="E8" s="5" t="inlineStr">
         <is>
+          <t>Person that made the cell, value should be in @classes with ID</t>
+        </is>
+      </c>
+      <c r="F8" s="5" t="inlineStr">
+        <is>
           <t>schema:creator</t>
-        </is>
-      </c>
-      <c r="F8" s="5" t="inlineStr">
-        <is>
-          <t>Person that made the cell, value should be in @classes with ID</t>
         </is>
       </c>
     </row>
@@ -784,12 +784,12 @@
           <t>recommended</t>
         </is>
       </c>
-      <c r="E9" s="4" t="inlineStr">
+      <c r="E9" s="4" t="n"/>
+      <c r="F9" s="4" t="inlineStr">
         <is>
           <t>rdfs:comment</t>
         </is>
       </c>
-      <c r="F9" s="4" t="n"/>
     </row>
     <row r="10">
       <c r="A10" s="5" t="inlineStr">
@@ -814,12 +814,12 @@
       </c>
       <c r="E10" s="5" t="inlineStr">
         <is>
+          <t>'manually' or 'by robot'</t>
+        </is>
+      </c>
+      <c r="F10" s="5" t="inlineStr">
+        <is>
           <t>rdfs:comment</t>
-        </is>
-      </c>
-      <c r="F10" s="5" t="inlineStr">
-        <is>
-          <t>'manually' or 'by robot'</t>
         </is>
       </c>
     </row>
@@ -846,12 +846,12 @@
       </c>
       <c r="E11" s="4" t="inlineStr">
         <is>
+          <t>Name of this schema, do not change</t>
+        </is>
+      </c>
+      <c r="F11" s="4" t="inlineStr">
+        <is>
           <t>rdfs:comment</t>
-        </is>
-      </c>
-      <c r="F11" s="4" t="inlineStr">
-        <is>
-          <t>Name of this schema, do not change</t>
         </is>
       </c>
     </row>
@@ -878,12 +878,12 @@
       </c>
       <c r="E12" s="5" t="inlineStr">
         <is>
+          <t>Version of this schema, do not change</t>
+        </is>
+      </c>
+      <c r="F12" s="5" t="inlineStr">
+        <is>
           <t>rdfs:comment</t>
-        </is>
-      </c>
-      <c r="F12" s="5" t="inlineStr">
-        <is>
-          <t>Version of this schema, do not change</t>
         </is>
       </c>
     </row>
@@ -920,12 +920,12 @@
           <t>required</t>
         </is>
       </c>
-      <c r="E14" s="4" t="inlineStr">
+      <c r="E14" s="4" t="n"/>
+      <c r="F14" s="4" t="inlineStr">
         <is>
           <t>hasPositiveElectrode-hasCurrentCollector</t>
         </is>
       </c>
-      <c r="F14" s="4" t="n"/>
     </row>
     <row r="15">
       <c r="A15" s="8" t="inlineStr">
@@ -946,12 +946,12 @@
           <t>recommended</t>
         </is>
       </c>
-      <c r="E15" s="8" t="inlineStr">
+      <c r="E15" s="8" t="n"/>
+      <c r="F15" s="8" t="inlineStr">
         <is>
           <t>hasPositiveElectrode-hasCurrentCollector-hasMeasuredProperty-Thickness</t>
         </is>
       </c>
-      <c r="F15" s="8" t="n"/>
     </row>
     <row r="16">
       <c r="A16" s="4" t="inlineStr">
@@ -974,12 +974,12 @@
           <t>required</t>
         </is>
       </c>
-      <c r="E16" s="4" t="inlineStr">
+      <c r="E16" s="4" t="n"/>
+      <c r="F16" s="4" t="inlineStr">
         <is>
           <t>hasPositiveElectrode-hasCoating-type|ElectrodeCoating-hasActiveMaterial</t>
         </is>
       </c>
-      <c r="F16" s="4" t="n"/>
     </row>
     <row r="17">
       <c r="A17" s="8" t="inlineStr">
@@ -1002,12 +1002,12 @@
           <t>recommended</t>
         </is>
       </c>
-      <c r="E17" s="8" t="inlineStr">
+      <c r="E17" s="8" t="n"/>
+      <c r="F17" s="8" t="inlineStr">
         <is>
           <t>hasPositiveElectrode-hasCoating-type|ElectrodeCoating-hasActiveMaterial-hasMeasuredProperty-type|molecularFormula-hasStringValue</t>
         </is>
       </c>
-      <c r="F17" s="8" t="n"/>
     </row>
     <row r="18">
       <c r="A18" s="4" t="inlineStr">
@@ -1028,12 +1028,12 @@
           <t>required</t>
         </is>
       </c>
-      <c r="E18" s="4" t="inlineStr">
+      <c r="E18" s="4" t="n"/>
+      <c r="F18" s="4" t="inlineStr">
         <is>
           <t>hasPositiveElectrode-hasCoating-type|ElectrodeCoating-hasActiveMaterial-hasMeasuredProperty-MassFraction</t>
         </is>
       </c>
-      <c r="F18" s="4" t="n"/>
     </row>
     <row r="19">
       <c r="A19" s="8" t="inlineStr">
@@ -1056,12 +1056,12 @@
           <t>required</t>
         </is>
       </c>
-      <c r="E19" s="8" t="inlineStr">
+      <c r="E19" s="8" t="n"/>
+      <c r="F19" s="8" t="inlineStr">
         <is>
           <t>hasPositiveElectrode-hasCoating-type|ElectrodeCoating-hasBinder</t>
         </is>
       </c>
-      <c r="F19" s="8" t="n"/>
     </row>
     <row r="20">
       <c r="A20" s="4" t="inlineStr">
@@ -1082,12 +1082,12 @@
           <t>required</t>
         </is>
       </c>
-      <c r="E20" s="4" t="inlineStr">
+      <c r="E20" s="4" t="n"/>
+      <c r="F20" s="4" t="inlineStr">
         <is>
           <t>hasPositiveElectrode-hasCoating-type|ElectrodeCoating-hasBinder-hasMeasuredProperty-MassFraction</t>
         </is>
       </c>
-      <c r="F20" s="4" t="n"/>
     </row>
     <row r="21">
       <c r="A21" s="8" t="inlineStr">
@@ -1110,12 +1110,12 @@
           <t>required</t>
         </is>
       </c>
-      <c r="E21" s="8" t="inlineStr">
+      <c r="E21" s="8" t="n"/>
+      <c r="F21" s="8" t="inlineStr">
         <is>
           <t>hasPositiveElectrode-hasCoating-type|ElectrodeCoating-hasConductiveAdditive</t>
         </is>
       </c>
-      <c r="F21" s="8" t="n"/>
     </row>
     <row r="22">
       <c r="A22" s="4" t="inlineStr">
@@ -1136,12 +1136,12 @@
           <t>required</t>
         </is>
       </c>
-      <c r="E22" s="4" t="inlineStr">
+      <c r="E22" s="4" t="n"/>
+      <c r="F22" s="4" t="inlineStr">
         <is>
           <t>hasPositiveElectrode-hasCoating-type|ElectrodeCoating-hasConductiveAdditive-hasMeasuredProperty-MassFraction</t>
         </is>
       </c>
-      <c r="F22" s="4" t="n"/>
     </row>
     <row r="23">
       <c r="A23" s="8" t="inlineStr">
@@ -1162,12 +1162,12 @@
           <t>required</t>
         </is>
       </c>
-      <c r="E23" s="8" t="inlineStr">
+      <c r="E23" s="8" t="n"/>
+      <c r="F23" s="8" t="inlineStr">
         <is>
           <t>hasPositiveElectrode-hasCoating-type|ElectrodeCoating-hasActiveMaterial-hasMeasuredProperty-MassLoading</t>
         </is>
       </c>
-      <c r="F23" s="8" t="n"/>
     </row>
     <row r="24">
       <c r="A24" s="4" t="inlineStr">
@@ -1188,12 +1188,12 @@
           <t>recommended</t>
         </is>
       </c>
-      <c r="E24" s="4" t="inlineStr">
+      <c r="E24" s="4" t="n"/>
+      <c r="F24" s="4" t="inlineStr">
         <is>
           <t>hasPositiveElectrode-hasCoating-type|ElectrodeCoating-hasMeasuredProperty-CalenderedCoatingThickness</t>
         </is>
       </c>
-      <c r="F24" s="4" t="n"/>
     </row>
     <row r="25">
       <c r="A25" s="9" t="inlineStr">
@@ -1226,12 +1226,12 @@
           <t>optional</t>
         </is>
       </c>
-      <c r="E26" s="4" t="inlineStr">
+      <c r="E26" s="4" t="n"/>
+      <c r="F26" s="4" t="inlineStr">
         <is>
           <t>hasPositiveElectrode-hasCoating-type|ElectrodeCoating-hasMeasuredProperty-Porosity</t>
         </is>
       </c>
-      <c r="F26" s="4" t="n"/>
     </row>
     <row r="27">
       <c r="A27" s="8" t="inlineStr">
@@ -1252,12 +1252,12 @@
           <t>optional</t>
         </is>
       </c>
-      <c r="E27" s="8" t="inlineStr">
+      <c r="E27" s="8" t="n"/>
+      <c r="F27" s="8" t="inlineStr">
         <is>
           <t>hasPositiveElectrode-hasCoating-type|ElectrodeCoating-hasMeasuredProperty-Tortuosity</t>
         </is>
       </c>
-      <c r="F27" s="8" t="n"/>
     </row>
     <row r="28">
       <c r="A28" s="4" t="inlineStr">
@@ -1278,12 +1278,12 @@
           <t>optional</t>
         </is>
       </c>
-      <c r="E28" s="4" t="inlineStr">
+      <c r="E28" s="4" t="n"/>
+      <c r="F28" s="4" t="inlineStr">
         <is>
           <t>hasPositiveElectrode-hasCoating-type|ElectrodeCoating-hasActiveMaterial-hasMeasuredProperty-D50ParticleSize</t>
         </is>
       </c>
-      <c r="F28" s="4" t="n"/>
     </row>
     <row r="29">
       <c r="A29" s="9" t="inlineStr">
@@ -1318,12 +1318,12 @@
           <t>optional</t>
         </is>
       </c>
-      <c r="E30" s="4" t="inlineStr">
+      <c r="E30" s="4" t="n"/>
+      <c r="F30" s="4" t="inlineStr">
         <is>
           <t>hasPositiveElectrode-hasMeasuredProperty-type|RatedCapacity-rev|hasOutput-type|Measurement-hasInput-ElectrochemicalHalfCell-rdfs:comment</t>
         </is>
       </c>
-      <c r="F30" s="4" t="n"/>
     </row>
     <row r="31">
       <c r="A31" s="8" t="inlineStr">
@@ -1346,12 +1346,12 @@
           <t>optional</t>
         </is>
       </c>
-      <c r="E31" s="8" t="inlineStr">
+      <c r="E31" s="8" t="n"/>
+      <c r="F31" s="8" t="inlineStr">
         <is>
           <t>hasPositiveElectrode-hasMeasuredProperty-type|RatedCapacity-rev|hasOutput-type|Measurement-hasInput-ElectrochemicalHalfCell-hasReferenceElectrode</t>
         </is>
       </c>
-      <c r="F31" s="8" t="n"/>
     </row>
     <row r="32">
       <c r="A32" s="4" t="inlineStr">
@@ -1372,12 +1372,12 @@
           <t>optional</t>
         </is>
       </c>
-      <c r="E32" s="4" t="inlineStr">
+      <c r="E32" s="4" t="n"/>
+      <c r="F32" s="4" t="inlineStr">
         <is>
           <t>hasPositiveElectrode-hasMeasuredProperty-type|RatedCapacity-rev|hasOutput-type|Measurement-hasInput-ConstantCurrentCharging-hasInput-LowerVoltageLimit</t>
         </is>
       </c>
-      <c r="F32" s="4" t="n"/>
     </row>
     <row r="33">
       <c r="A33" s="8" t="inlineStr">
@@ -1398,12 +1398,12 @@
           <t>optional</t>
         </is>
       </c>
-      <c r="E33" s="8" t="inlineStr">
+      <c r="E33" s="8" t="n"/>
+      <c r="F33" s="8" t="inlineStr">
         <is>
           <t>hasPositiveElectrode-hasMeasuredProperty-type|RatedCapacity-rev|hasOutput-type|Measurement-hasInput-ConstantCurrentCharging-hasInput-ElectricCurrentDensity</t>
         </is>
       </c>
-      <c r="F33" s="8" t="n"/>
     </row>
     <row r="34">
       <c r="A34" s="4" t="inlineStr">
@@ -1424,12 +1424,12 @@
           <t>optional</t>
         </is>
       </c>
-      <c r="E34" s="4" t="inlineStr">
+      <c r="E34" s="4" t="n"/>
+      <c r="F34" s="4" t="inlineStr">
         <is>
           <t>hasPositiveElectrode-hasMeasuredProperty-type|RatedCapacity-rev|hasOutput-type|Measurement-hasInput-ConstantCurrentCharging-hasInput-UpperVoltageLimit</t>
         </is>
       </c>
-      <c r="F34" s="4" t="n"/>
     </row>
     <row r="35">
       <c r="A35" s="8" t="inlineStr">
@@ -1450,12 +1450,12 @@
           <t>optional</t>
         </is>
       </c>
-      <c r="E35" s="8" t="inlineStr">
+      <c r="E35" s="8" t="n"/>
+      <c r="F35" s="8" t="inlineStr">
         <is>
           <t>hasPositiveElectrode-hasMeasuredProperty-type|RatedCapacity-rev|hasOutput-type|Measurement-hasInput-ConstantVoltageCharging-hasInput-UpperVoltageLimit</t>
         </is>
       </c>
-      <c r="F35" s="8" t="n"/>
     </row>
     <row r="36">
       <c r="A36" s="4" t="inlineStr">
@@ -1476,12 +1476,12 @@
           <t>optional</t>
         </is>
       </c>
-      <c r="E36" s="4" t="inlineStr">
+      <c r="E36" s="4" t="n"/>
+      <c r="F36" s="4" t="inlineStr">
         <is>
           <t>hasPositiveElectrode-hasMeasuredProperty-type|RatedCapacity-rev|hasOutput-type|Measurement-hasInput-ConstantVoltageCharging-hasInput-LowerCurrentDensityLimit</t>
         </is>
       </c>
-      <c r="F36" s="4" t="n"/>
     </row>
     <row r="37">
       <c r="A37" s="8" t="inlineStr">
@@ -1502,12 +1502,12 @@
           <t>optional</t>
         </is>
       </c>
-      <c r="E37" s="8" t="inlineStr">
+      <c r="E37" s="8" t="n"/>
+      <c r="F37" s="8" t="inlineStr">
         <is>
           <t>hasPositiveElectrode-hasMeasuredProperty-type|RatedCapacity-rev|hasOutput-type|Measurement-hasInput-ConstantCurrentDischarging-hasInput-UpperVoltageLimit</t>
         </is>
       </c>
-      <c r="F37" s="8" t="n"/>
     </row>
     <row r="38">
       <c r="A38" s="4" t="inlineStr">
@@ -1528,12 +1528,12 @@
           <t>optional</t>
         </is>
       </c>
-      <c r="E38" s="4" t="inlineStr">
+      <c r="E38" s="4" t="n"/>
+      <c r="F38" s="4" t="inlineStr">
         <is>
           <t>hasPositiveElectrode-hasMeasuredProperty-type|RatedCapacity-rev|hasOutput-type|Measurement-hasInput-ConstantCurrentDischarging-hasInput-ElectricCurrentDensity</t>
         </is>
       </c>
-      <c r="F38" s="4" t="n"/>
     </row>
     <row r="39">
       <c r="A39" s="8" t="inlineStr">
@@ -1554,12 +1554,12 @@
           <t>optional</t>
         </is>
       </c>
-      <c r="E39" s="8" t="inlineStr">
+      <c r="E39" s="8" t="n"/>
+      <c r="F39" s="8" t="inlineStr">
         <is>
           <t>hasPositiveElectrode-hasMeasuredProperty-type|RatedCapacity-rev|hasOutput-type|Measurement-hasInput-ConstantCurrentDischarging-hasInput-LowerVoltageLimit</t>
         </is>
       </c>
-      <c r="F39" s="8" t="n"/>
     </row>
     <row r="40">
       <c r="A40" s="4" t="inlineStr">
@@ -1580,12 +1580,12 @@
           <t>optional</t>
         </is>
       </c>
-      <c r="E40" s="4" t="inlineStr">
+      <c r="E40" s="4" t="n"/>
+      <c r="F40" s="4" t="inlineStr">
         <is>
           <t>hasPositiveElectrode-hasMeasuredProperty-type|RatedCapacity-rev|hasOutput-type|Measurement-hasInput-ConstantVoltageCharging-hasInput-LowerVoltageLimit</t>
         </is>
       </c>
-      <c r="F40" s="4" t="n"/>
     </row>
     <row r="41">
       <c r="A41" s="8" t="inlineStr">
@@ -1606,12 +1606,12 @@
           <t>optional</t>
         </is>
       </c>
-      <c r="E41" s="8" t="inlineStr">
+      <c r="E41" s="8" t="n"/>
+      <c r="F41" s="8" t="inlineStr">
         <is>
           <t>hasPositiveElectrode-hasMeasuredProperty-type|RatedCapacity</t>
         </is>
       </c>
-      <c r="F41" s="8" t="n"/>
     </row>
     <row r="42">
       <c r="A42" s="4" t="inlineStr">
@@ -1632,12 +1632,12 @@
           <t>optional</t>
         </is>
       </c>
-      <c r="E42" s="4" t="inlineStr">
+      <c r="E42" s="4" t="n"/>
+      <c r="F42" s="4" t="inlineStr">
         <is>
           <t>hasPositiveElectrode-hasMeasuredProperty-type|RatedCapacity</t>
         </is>
       </c>
-      <c r="F42" s="4" t="n"/>
     </row>
     <row r="43">
       <c r="A43" s="9" t="inlineStr">
@@ -1672,12 +1672,12 @@
           <t>optional</t>
         </is>
       </c>
-      <c r="E44" s="4" t="inlineStr">
+      <c r="E44" s="4" t="n"/>
+      <c r="F44" s="4" t="inlineStr">
         <is>
           <t>hasPositiveElectrode-schema:manufacturer</t>
         </is>
       </c>
-      <c r="F44" s="4" t="n"/>
     </row>
     <row r="45">
       <c r="A45" s="8" t="inlineStr">
@@ -1698,12 +1698,12 @@
           <t>optional</t>
         </is>
       </c>
-      <c r="E45" s="8" t="inlineStr">
+      <c r="E45" s="8" t="n"/>
+      <c r="F45" s="8" t="inlineStr">
         <is>
           <t>hasPositiveElectrode-schema:productID</t>
         </is>
       </c>
-      <c r="F45" s="8" t="n"/>
     </row>
     <row r="46">
       <c r="A46" s="4" t="inlineStr">
@@ -1722,12 +1722,12 @@
           <t>optional</t>
         </is>
       </c>
-      <c r="E46" s="4" t="inlineStr">
+      <c r="E46" s="4" t="n"/>
+      <c r="F46" s="4" t="inlineStr">
         <is>
           <t>hasPositiveElectrode-hasCurrentCollector-schema:manufacturer</t>
         </is>
       </c>
-      <c r="F46" s="4" t="n"/>
     </row>
     <row r="47">
       <c r="A47" s="8" t="inlineStr">
@@ -1746,12 +1746,12 @@
           <t>optional</t>
         </is>
       </c>
-      <c r="E47" s="8" t="inlineStr">
+      <c r="E47" s="8" t="n"/>
+      <c r="F47" s="8" t="inlineStr">
         <is>
           <t>hasPositiveElectrode-hasCurrentCollector-schema:productID</t>
         </is>
       </c>
-      <c r="F47" s="8" t="n"/>
     </row>
     <row r="48">
       <c r="A48" s="4" t="inlineStr">
@@ -1770,12 +1770,12 @@
           <t>optional</t>
         </is>
       </c>
-      <c r="E48" s="4" t="inlineStr">
+      <c r="E48" s="4" t="n"/>
+      <c r="F48" s="4" t="inlineStr">
         <is>
           <t>hasPositiveElectrode-hasCoating-type|ElectrodeCoating-hasActiveMaterial-schema:manufacturer</t>
         </is>
       </c>
-      <c r="F48" s="4" t="n"/>
     </row>
     <row r="49">
       <c r="A49" s="8" t="inlineStr">
@@ -1794,12 +1794,12 @@
           <t>optional</t>
         </is>
       </c>
-      <c r="E49" s="8" t="inlineStr">
+      <c r="E49" s="8" t="n"/>
+      <c r="F49" s="8" t="inlineStr">
         <is>
           <t>hasPositiveElectrode-hasCoating-type|ElectrodeCoating-hasActiveMaterial-schema:productID</t>
         </is>
       </c>
-      <c r="F49" s="8" t="n"/>
     </row>
     <row r="50">
       <c r="A50" s="4" t="inlineStr">
@@ -1818,12 +1818,12 @@
           <t>optional</t>
         </is>
       </c>
-      <c r="E50" s="4" t="inlineStr">
+      <c r="E50" s="4" t="n"/>
+      <c r="F50" s="4" t="inlineStr">
         <is>
           <t>hasPositiveElectrode-hasCoating-type|ElectrodeCoating-hasBinder-schema:manufacturer</t>
         </is>
       </c>
-      <c r="F50" s="4" t="n"/>
     </row>
     <row r="51">
       <c r="A51" s="8" t="inlineStr">
@@ -1842,12 +1842,12 @@
           <t>optional</t>
         </is>
       </c>
-      <c r="E51" s="8" t="inlineStr">
+      <c r="E51" s="8" t="n"/>
+      <c r="F51" s="8" t="inlineStr">
         <is>
           <t>hasPositiveElectrode-hasCoating-type|ElectrodeCoating-hasBinder-schema:productID</t>
         </is>
       </c>
-      <c r="F51" s="8" t="n"/>
     </row>
     <row r="52">
       <c r="A52" s="4" t="inlineStr">
@@ -1866,12 +1866,12 @@
           <t>optional</t>
         </is>
       </c>
-      <c r="E52" s="4" t="inlineStr">
+      <c r="E52" s="4" t="n"/>
+      <c r="F52" s="4" t="inlineStr">
         <is>
           <t>hasPositiveElectrode-hasCoating-type|ElectrodeCoating-hasConductiveAdditive-schema:manufacturer</t>
         </is>
       </c>
-      <c r="F52" s="4" t="n"/>
     </row>
     <row r="53">
       <c r="A53" s="8" t="inlineStr">
@@ -1890,12 +1890,12 @@
           <t>optional</t>
         </is>
       </c>
-      <c r="E53" s="8" t="inlineStr">
+      <c r="E53" s="8" t="n"/>
+      <c r="F53" s="8" t="inlineStr">
         <is>
           <t>hasPositiveElectrode-hasCoating-type|ElectrodeCoating-hasConductiveAdditive-schema:productID</t>
         </is>
       </c>
-      <c r="F53" s="8" t="n"/>
     </row>
     <row r="54">
       <c r="A54" s="10" t="inlineStr">
@@ -1930,12 +1930,12 @@
           <t>required</t>
         </is>
       </c>
-      <c r="E55" s="4" t="inlineStr">
+      <c r="E55" s="4" t="n"/>
+      <c r="F55" s="4" t="inlineStr">
         <is>
           <t>hasNegativeElectrode-hasCurrentCollector</t>
         </is>
       </c>
-      <c r="F55" s="4" t="n"/>
     </row>
     <row r="56">
       <c r="A56" s="12" t="inlineStr">
@@ -1956,12 +1956,12 @@
           <t>recommended</t>
         </is>
       </c>
-      <c r="E56" s="12" t="inlineStr">
+      <c r="E56" s="12" t="n"/>
+      <c r="F56" s="12" t="inlineStr">
         <is>
           <t>hasNegativeElectrode-hasCurrentCollector-hasMeasuredProperty-Thickness</t>
         </is>
       </c>
-      <c r="F56" s="12" t="n"/>
     </row>
     <row r="57">
       <c r="A57" s="4" t="inlineStr">
@@ -1984,12 +1984,12 @@
           <t>required</t>
         </is>
       </c>
-      <c r="E57" s="4" t="inlineStr">
+      <c r="E57" s="4" t="n"/>
+      <c r="F57" s="4" t="inlineStr">
         <is>
           <t>hasNegativeElectrode-hasCoating-type|ElectrodeCoating-hasActiveMaterial</t>
         </is>
       </c>
-      <c r="F57" s="4" t="n"/>
     </row>
     <row r="58">
       <c r="A58" s="12" t="inlineStr">
@@ -2010,12 +2010,12 @@
           <t>required</t>
         </is>
       </c>
-      <c r="E58" s="12" t="inlineStr">
+      <c r="E58" s="12" t="n"/>
+      <c r="F58" s="12" t="inlineStr">
         <is>
           <t>hasNegativeElectrode-hasCoating-type|ElectrodeCoating-hasActiveMaterial-hasMeasuredProperty-MassFraction</t>
         </is>
       </c>
-      <c r="F58" s="12" t="n"/>
     </row>
     <row r="59">
       <c r="A59" s="4" t="inlineStr">
@@ -2038,12 +2038,12 @@
           <t>required</t>
         </is>
       </c>
-      <c r="E59" s="4" t="inlineStr">
+      <c r="E59" s="4" t="n"/>
+      <c r="F59" s="4" t="inlineStr">
         <is>
           <t>hasNegativeElectrode-hasCoating-type|ElectrodeCoating-hasBinder</t>
         </is>
       </c>
-      <c r="F59" s="4" t="n"/>
     </row>
     <row r="60">
       <c r="A60" s="12" t="inlineStr">
@@ -2064,12 +2064,12 @@
           <t>required</t>
         </is>
       </c>
-      <c r="E60" s="12" t="inlineStr">
+      <c r="E60" s="12" t="n"/>
+      <c r="F60" s="12" t="inlineStr">
         <is>
           <t>hasNegativeElectrode-hasCoating-type|ElectrodeCoating-hasBinder-hasMeasuredProperty-MassFraction</t>
         </is>
       </c>
-      <c r="F60" s="12" t="n"/>
     </row>
     <row r="61">
       <c r="A61" s="4" t="inlineStr">
@@ -2092,12 +2092,12 @@
           <t>required</t>
         </is>
       </c>
-      <c r="E61" s="4" t="inlineStr">
+      <c r="E61" s="4" t="n"/>
+      <c r="F61" s="4" t="inlineStr">
         <is>
           <t>hasNegativeElectrode-hasCoating-type|ElectrodeCoating-hasConductiveAdditive</t>
         </is>
       </c>
-      <c r="F61" s="4" t="n"/>
     </row>
     <row r="62">
       <c r="A62" s="12" t="inlineStr">
@@ -2118,12 +2118,12 @@
           <t>required</t>
         </is>
       </c>
-      <c r="E62" s="12" t="inlineStr">
+      <c r="E62" s="12" t="n"/>
+      <c r="F62" s="12" t="inlineStr">
         <is>
           <t>hasNegativeElectrode-hasCoating-type|ElectrodeCoating-hasConductiveAdditive-hasMeasuredProperty-MassFraction</t>
         </is>
       </c>
-      <c r="F62" s="12" t="n"/>
     </row>
     <row r="63">
       <c r="A63" s="4" t="inlineStr">
@@ -2144,12 +2144,12 @@
           <t>required</t>
         </is>
       </c>
-      <c r="E63" s="4" t="inlineStr">
+      <c r="E63" s="4" t="n"/>
+      <c r="F63" s="4" t="inlineStr">
         <is>
           <t>hasNegativeElectrode-hasCoating-type|ElectrodeCoating-hasActiveMaterial-hasMeasuredProperty-MassLoading</t>
         </is>
       </c>
-      <c r="F63" s="4" t="n"/>
     </row>
     <row r="64">
       <c r="A64" s="12" t="inlineStr">
@@ -2170,12 +2170,12 @@
           <t>recommended</t>
         </is>
       </c>
-      <c r="E64" s="12" t="inlineStr">
+      <c r="E64" s="12" t="n"/>
+      <c r="F64" s="12" t="inlineStr">
         <is>
           <t>hasNegativeElectrode-hasCoating-type|ElectrodeCoating-hasMeasuredProperty-CalenderedCoatingThickness</t>
         </is>
       </c>
-      <c r="F64" s="12" t="n"/>
     </row>
     <row r="65">
       <c r="A65" s="13" t="inlineStr">
@@ -2208,12 +2208,12 @@
           <t>optional</t>
         </is>
       </c>
-      <c r="E66" s="4" t="inlineStr">
+      <c r="E66" s="4" t="n"/>
+      <c r="F66" s="4" t="inlineStr">
         <is>
           <t>hasNegativeElectrode-hasCoating-type|ElectrodeCoating-hasMeasuredProperty-Porosity</t>
         </is>
       </c>
-      <c r="F66" s="4" t="n"/>
     </row>
     <row r="67">
       <c r="A67" s="12" t="inlineStr">
@@ -2234,12 +2234,12 @@
           <t>optional</t>
         </is>
       </c>
-      <c r="E67" s="12" t="inlineStr">
+      <c r="E67" s="12" t="n"/>
+      <c r="F67" s="12" t="inlineStr">
         <is>
           <t>hasNegativeElectrode-hasCoating-type|ElectrodeCoating-hasMeasuredProperty-Tortuosity</t>
         </is>
       </c>
-      <c r="F67" s="12" t="n"/>
     </row>
     <row r="68">
       <c r="A68" s="4" t="inlineStr">
@@ -2260,12 +2260,12 @@
           <t>optional</t>
         </is>
       </c>
-      <c r="E68" s="4" t="inlineStr">
+      <c r="E68" s="4" t="n"/>
+      <c r="F68" s="4" t="inlineStr">
         <is>
           <t>hasNegativeElectrode-hasCoating-type|ElectrodeCoating-hasActiveMaterial-hasMeasuredProperty-D50ParticleSize</t>
         </is>
       </c>
-      <c r="F68" s="4" t="n"/>
     </row>
     <row r="69">
       <c r="A69" s="13" t="inlineStr">
@@ -2300,12 +2300,12 @@
           <t>optional</t>
         </is>
       </c>
-      <c r="E70" s="4" t="inlineStr">
+      <c r="E70" s="4" t="n"/>
+      <c r="F70" s="4" t="inlineStr">
         <is>
           <t>hasNegativeElectrode-hasMeasuredProperty-type|RatedCapacity-rev|hasOutput-type|Measurement-hasInput-ElectrochemicalHalfCell-rdfs:comment</t>
         </is>
       </c>
-      <c r="F70" s="4" t="n"/>
     </row>
     <row r="71">
       <c r="A71" s="12" t="inlineStr">
@@ -2328,12 +2328,12 @@
           <t>optional</t>
         </is>
       </c>
-      <c r="E71" s="12" t="inlineStr">
+      <c r="E71" s="12" t="n"/>
+      <c r="F71" s="12" t="inlineStr">
         <is>
           <t>hasNegativeElectrode-hasMeasuredProperty-type|RatedCapacity-rev|hasOutput-type|Measurement-hasInput-ElectrochemicalHalfCell-hasReferenceElectrode</t>
         </is>
       </c>
-      <c r="F71" s="12" t="n"/>
     </row>
     <row r="72">
       <c r="A72" s="4" t="inlineStr">
@@ -2354,12 +2354,12 @@
           <t>optional</t>
         </is>
       </c>
-      <c r="E72" s="4" t="inlineStr">
+      <c r="E72" s="4" t="n"/>
+      <c r="F72" s="4" t="inlineStr">
         <is>
           <t>hasNegativeElectrode-hasMeasuredProperty-type|RatedCapacity-rev|hasOutput-type|Measurement-hasInput-ConstantCurrentCharging-hasInput-UpperVoltageLimit</t>
         </is>
       </c>
-      <c r="F72" s="4" t="n"/>
     </row>
     <row r="73">
       <c r="A73" s="12" t="inlineStr">
@@ -2380,12 +2380,12 @@
           <t>optional</t>
         </is>
       </c>
-      <c r="E73" s="12" t="inlineStr">
+      <c r="E73" s="12" t="n"/>
+      <c r="F73" s="12" t="inlineStr">
         <is>
           <t>hasNegativeElectrode-hasMeasuredProperty-type|RatedCapacity-rev|hasOutput-type|Measurement-hasInput-ConstantCurrentCharging-hasInput-ElectricCurrentDensity</t>
         </is>
       </c>
-      <c r="F73" s="12" t="n"/>
     </row>
     <row r="74">
       <c r="A74" s="4" t="inlineStr">
@@ -2406,12 +2406,12 @@
           <t>optional</t>
         </is>
       </c>
-      <c r="E74" s="4" t="inlineStr">
+      <c r="E74" s="4" t="n"/>
+      <c r="F74" s="4" t="inlineStr">
         <is>
           <t>hasNegativeElectrode-hasMeasuredProperty-type|RatedCapacity-rev|hasOutput-type|Measurement-hasInput-ConstantCurrentCharging-hasInput-LowerVoltageLimit</t>
         </is>
       </c>
-      <c r="F74" s="4" t="n"/>
     </row>
     <row r="75">
       <c r="A75" s="12" t="inlineStr">
@@ -2432,12 +2432,12 @@
           <t>optional</t>
         </is>
       </c>
-      <c r="E75" s="12" t="inlineStr">
+      <c r="E75" s="12" t="n"/>
+      <c r="F75" s="12" t="inlineStr">
         <is>
           <t>hasNegativeElectrode-hasMeasuredProperty-type|RatedCapacity-rev|hasOutput-type|Measurement-hasInput-ConstantVoltageCharging-hasInput-LowerVoltageLimit</t>
         </is>
       </c>
-      <c r="F75" s="12" t="n"/>
     </row>
     <row r="76">
       <c r="A76" s="4" t="inlineStr">
@@ -2458,12 +2458,12 @@
           <t>optional</t>
         </is>
       </c>
-      <c r="E76" s="4" t="inlineStr">
+      <c r="E76" s="4" t="n"/>
+      <c r="F76" s="4" t="inlineStr">
         <is>
           <t>hasNegativeElectrode-hasMeasuredProperty-type|RatedCapacity-rev|hasOutput-type|Measurement-hasInput-ConstantVoltageCharging-hasInput-LowerCurrentDensityLimit</t>
         </is>
       </c>
-      <c r="F76" s="4" t="n"/>
     </row>
     <row r="77">
       <c r="A77" s="12" t="inlineStr">
@@ -2484,12 +2484,12 @@
           <t>optional</t>
         </is>
       </c>
-      <c r="E77" s="12" t="inlineStr">
+      <c r="E77" s="12" t="n"/>
+      <c r="F77" s="12" t="inlineStr">
         <is>
           <t>hasNegativeElectrode-hasMeasuredProperty-type|RatedCapacity-rev|hasOutput-type|Measurement-hasInput-ConstantCurrentDischarging-hasInput-LowerVoltageLimit</t>
         </is>
       </c>
-      <c r="F77" s="12" t="n"/>
     </row>
     <row r="78">
       <c r="A78" s="4" t="inlineStr">
@@ -2510,12 +2510,12 @@
           <t>optional</t>
         </is>
       </c>
-      <c r="E78" s="4" t="inlineStr">
+      <c r="E78" s="4" t="n"/>
+      <c r="F78" s="4" t="inlineStr">
         <is>
           <t>hasNegativeElectrode-hasMeasuredProperty-type|RatedCapacity-rev|hasOutput-type|Measurement-hasInput-ConstantCurrentDischarging-hasInput-ElectricCurrentDensity</t>
         </is>
       </c>
-      <c r="F78" s="4" t="n"/>
     </row>
     <row r="79">
       <c r="A79" s="12" t="inlineStr">
@@ -2536,12 +2536,12 @@
           <t>optional</t>
         </is>
       </c>
-      <c r="E79" s="12" t="inlineStr">
+      <c r="E79" s="12" t="n"/>
+      <c r="F79" s="12" t="inlineStr">
         <is>
           <t>hasNegativeElectrode-hasMeasuredProperty-type|RatedCapacity-rev|hasOutput-type|Measurement-hasInput-ConstantCurrentDischarging-hasInput-UpperVoltageLimit</t>
         </is>
       </c>
-      <c r="F79" s="12" t="n"/>
     </row>
     <row r="80">
       <c r="A80" s="4" t="inlineStr">
@@ -2562,12 +2562,12 @@
           <t>optional</t>
         </is>
       </c>
-      <c r="E80" s="4" t="inlineStr">
+      <c r="E80" s="4" t="n"/>
+      <c r="F80" s="4" t="inlineStr">
         <is>
           <t>hasNegativeElectrode-hasMeasuredProperty-type|RatedCapacity-rev|hasOutput-type|Measurement-hasInput-ConstantVoltageCharging-hasInput-UpperVoltageLimit</t>
         </is>
       </c>
-      <c r="F80" s="4" t="n"/>
     </row>
     <row r="81">
       <c r="A81" s="12" t="inlineStr">
@@ -2588,12 +2588,12 @@
           <t>optional</t>
         </is>
       </c>
-      <c r="E81" s="12" t="inlineStr">
+      <c r="E81" s="12" t="n"/>
+      <c r="F81" s="12" t="inlineStr">
         <is>
           <t>hasNegativeElectrode-hasMeasuredProperty-type|RatedCapacity</t>
         </is>
       </c>
-      <c r="F81" s="12" t="n"/>
     </row>
     <row r="82">
       <c r="A82" s="4" t="inlineStr">
@@ -2614,12 +2614,12 @@
           <t>optional</t>
         </is>
       </c>
-      <c r="E82" s="4" t="inlineStr">
+      <c r="E82" s="4" t="n"/>
+      <c r="F82" s="4" t="inlineStr">
         <is>
           <t>hasNegativeElectrode-hasMeasuredProperty-type|RatedCapacity</t>
         </is>
       </c>
-      <c r="F82" s="4" t="n"/>
     </row>
     <row r="83">
       <c r="A83" s="13" t="inlineStr">
@@ -2654,12 +2654,12 @@
           <t>optional</t>
         </is>
       </c>
-      <c r="E84" s="4" t="inlineStr">
+      <c r="E84" s="4" t="n"/>
+      <c r="F84" s="4" t="inlineStr">
         <is>
           <t>hasNegativeElectrode-schema:manufacturer</t>
         </is>
       </c>
-      <c r="F84" s="4" t="n"/>
     </row>
     <row r="85">
       <c r="A85" s="12" t="inlineStr">
@@ -2682,12 +2682,12 @@
           <t>optional</t>
         </is>
       </c>
-      <c r="E85" s="12" t="inlineStr">
+      <c r="E85" s="12" t="n"/>
+      <c r="F85" s="12" t="inlineStr">
         <is>
           <t>hasNegativeElectrode-schema:productID</t>
         </is>
       </c>
-      <c r="F85" s="12" t="n"/>
     </row>
     <row r="86">
       <c r="A86" s="4" t="inlineStr">
@@ -2706,12 +2706,12 @@
           <t>optional</t>
         </is>
       </c>
-      <c r="E86" s="4" t="inlineStr">
+      <c r="E86" s="4" t="n"/>
+      <c r="F86" s="4" t="inlineStr">
         <is>
           <t>hasNegativeElectrode-hasCurrentCollector-schema:manufacturer</t>
         </is>
       </c>
-      <c r="F86" s="4" t="n"/>
     </row>
     <row r="87">
       <c r="A87" s="12" t="inlineStr">
@@ -2730,12 +2730,12 @@
           <t>optional</t>
         </is>
       </c>
-      <c r="E87" s="12" t="inlineStr">
+      <c r="E87" s="12" t="n"/>
+      <c r="F87" s="12" t="inlineStr">
         <is>
           <t>hasNegativeElectrode-hasCurrentCollector-schema:productID</t>
         </is>
       </c>
-      <c r="F87" s="12" t="n"/>
     </row>
     <row r="88">
       <c r="A88" s="4" t="inlineStr">
@@ -2754,12 +2754,12 @@
           <t>optional</t>
         </is>
       </c>
-      <c r="E88" s="4" t="inlineStr">
+      <c r="E88" s="4" t="n"/>
+      <c r="F88" s="4" t="inlineStr">
         <is>
           <t>hasNegativeElectrode-hasCoating-type|ElectrodeCoating-hasActiveMaterial-schema:manufacturer</t>
         </is>
       </c>
-      <c r="F88" s="4" t="n"/>
     </row>
     <row r="89">
       <c r="A89" s="12" t="inlineStr">
@@ -2778,12 +2778,12 @@
           <t>optional</t>
         </is>
       </c>
-      <c r="E89" s="12" t="inlineStr">
+      <c r="E89" s="12" t="n"/>
+      <c r="F89" s="12" t="inlineStr">
         <is>
           <t>hasNegativeElectrode-hasCoating-type|ElectrodeCoating-hasActiveMaterial-schema:productID</t>
         </is>
       </c>
-      <c r="F89" s="12" t="n"/>
     </row>
     <row r="90">
       <c r="A90" s="4" t="inlineStr">
@@ -2802,12 +2802,12 @@
           <t>optional</t>
         </is>
       </c>
-      <c r="E90" s="4" t="inlineStr">
+      <c r="E90" s="4" t="n"/>
+      <c r="F90" s="4" t="inlineStr">
         <is>
           <t>hasNegativeElectrode-hasCoating-type|ElectrodeCoating-hasBinder-schema:manufacturer</t>
         </is>
       </c>
-      <c r="F90" s="4" t="n"/>
     </row>
     <row r="91">
       <c r="A91" s="12" t="inlineStr">
@@ -2826,12 +2826,12 @@
           <t>optional</t>
         </is>
       </c>
-      <c r="E91" s="12" t="inlineStr">
+      <c r="E91" s="12" t="n"/>
+      <c r="F91" s="12" t="inlineStr">
         <is>
           <t>hasNegativeElectrode-hasCoating-type|ElectrodeCoating-hasBinder-schema:productID</t>
         </is>
       </c>
-      <c r="F91" s="12" t="n"/>
     </row>
     <row r="92">
       <c r="A92" s="4" t="inlineStr">
@@ -2850,12 +2850,12 @@
           <t>optional</t>
         </is>
       </c>
-      <c r="E92" s="4" t="inlineStr">
+      <c r="E92" s="4" t="n"/>
+      <c r="F92" s="4" t="inlineStr">
         <is>
           <t>hasNegativeElectrode-hasCoating-type|ElectrodeCoating-hasConductiveAdditive-schema:manufacturer</t>
         </is>
       </c>
-      <c r="F92" s="4" t="n"/>
     </row>
     <row r="93">
       <c r="A93" s="12" t="inlineStr">
@@ -2874,12 +2874,12 @@
           <t>optional</t>
         </is>
       </c>
-      <c r="E93" s="12" t="inlineStr">
+      <c r="E93" s="12" t="n"/>
+      <c r="F93" s="12" t="inlineStr">
         <is>
           <t>hasNegativeElectrode-hasCoating-type|ElectrodeCoating-hasConductiveAdditive-schema:productID</t>
         </is>
       </c>
-      <c r="F93" s="12" t="n"/>
     </row>
     <row r="94">
       <c r="A94" s="14" t="inlineStr">
@@ -2914,12 +2914,12 @@
           <t>required</t>
         </is>
       </c>
-      <c r="E95" s="4" t="inlineStr">
+      <c r="E95" s="4" t="n"/>
+      <c r="F95" s="4" t="inlineStr">
         <is>
           <t>hasElectrolyte-hasSolvent-hasConstituentA</t>
         </is>
       </c>
-      <c r="F95" s="4" t="n"/>
     </row>
     <row r="96">
       <c r="A96" s="16" t="inlineStr">
@@ -2940,12 +2940,12 @@
           <t>required</t>
         </is>
       </c>
-      <c r="E96" s="16" t="inlineStr">
+      <c r="E96" s="16" t="n"/>
+      <c r="F96" s="16" t="inlineStr">
         <is>
           <t>hasElectrolyte-hasSolvent-hasConstituentA-hasMeasuredProperty-VolumeFraction</t>
         </is>
       </c>
-      <c r="F96" s="16" t="n"/>
     </row>
     <row r="97">
       <c r="A97" s="4" t="inlineStr">
@@ -2968,12 +2968,12 @@
           <t>recommended</t>
         </is>
       </c>
-      <c r="E97" s="4" t="inlineStr">
+      <c r="E97" s="4" t="n"/>
+      <c r="F97" s="4" t="inlineStr">
         <is>
           <t>hasElectrolyte-hasSolvent-hasConstituentB</t>
         </is>
       </c>
-      <c r="F97" s="4" t="n"/>
     </row>
     <row r="98">
       <c r="A98" s="16" t="inlineStr">
@@ -2994,12 +2994,12 @@
           <t>recommended</t>
         </is>
       </c>
-      <c r="E98" s="16" t="inlineStr">
+      <c r="E98" s="16" t="n"/>
+      <c r="F98" s="16" t="inlineStr">
         <is>
           <t>hasElectrolyte-hasSolvent-hasConstituentB-hasMeasuredProperty-VolumeFraction</t>
         </is>
       </c>
-      <c r="F98" s="16" t="n"/>
     </row>
     <row r="99">
       <c r="A99" s="4" t="inlineStr">
@@ -3022,12 +3022,12 @@
           <t>required</t>
         </is>
       </c>
-      <c r="E99" s="4" t="inlineStr">
+      <c r="E99" s="4" t="n"/>
+      <c r="F99" s="4" t="inlineStr">
         <is>
           <t>hasElectrolyte-hasSolute-hasConstituentA</t>
         </is>
       </c>
-      <c r="F99" s="4" t="n"/>
     </row>
     <row r="100">
       <c r="A100" s="16" t="inlineStr">
@@ -3048,12 +3048,12 @@
           <t>required</t>
         </is>
       </c>
-      <c r="E100" s="16" t="inlineStr">
+      <c r="E100" s="16" t="n"/>
+      <c r="F100" s="16" t="inlineStr">
         <is>
           <t>hasElectrolyte-hasSolute-hasConstituentA-hasMeasuredProperty-AmountConcentration</t>
         </is>
       </c>
-      <c r="F100" s="16" t="n"/>
     </row>
     <row r="101">
       <c r="A101" s="4" t="inlineStr">
@@ -3076,12 +3076,12 @@
           <t>optional</t>
         </is>
       </c>
-      <c r="E101" s="4" t="inlineStr">
+      <c r="E101" s="4" t="n"/>
+      <c r="F101" s="4" t="inlineStr">
         <is>
           <t>hasElectrolyte-hasSolute-hasConstituentB</t>
         </is>
       </c>
-      <c r="F101" s="4" t="n"/>
     </row>
     <row r="102">
       <c r="A102" s="16" t="inlineStr">
@@ -3102,12 +3102,12 @@
           <t>optional</t>
         </is>
       </c>
-      <c r="E102" s="16" t="inlineStr">
+      <c r="E102" s="16" t="n"/>
+      <c r="F102" s="16" t="inlineStr">
         <is>
           <t>hasElectrolyte-hasSolute-hasConstituentB-hasMeasuredProperty-AmountConcentration</t>
         </is>
       </c>
-      <c r="F102" s="16" t="n"/>
     </row>
     <row r="103">
       <c r="A103" s="4" t="inlineStr">
@@ -3130,12 +3130,12 @@
           <t>optional</t>
         </is>
       </c>
-      <c r="E103" s="4" t="inlineStr">
+      <c r="E103" s="4" t="n"/>
+      <c r="F103" s="4" t="inlineStr">
         <is>
           <t>hasElectrolyte-hasSolute-hasAdditive-hasConstituentA</t>
         </is>
       </c>
-      <c r="F103" s="4" t="n"/>
     </row>
     <row r="104">
       <c r="A104" s="16" t="inlineStr">
@@ -3156,12 +3156,12 @@
           <t>optional</t>
         </is>
       </c>
-      <c r="E104" s="16" t="inlineStr">
+      <c r="E104" s="16" t="n"/>
+      <c r="F104" s="16" t="inlineStr">
         <is>
           <t>hasElectrolyte-hasSolute-hasAdditive-hasConstituentA-hasMeasuredProperty-AmountConcentration</t>
         </is>
       </c>
-      <c r="F104" s="16" t="n"/>
     </row>
     <row r="105">
       <c r="A105" s="4" t="inlineStr">
@@ -3184,12 +3184,12 @@
           <t>optional</t>
         </is>
       </c>
-      <c r="E105" s="4" t="inlineStr">
+      <c r="E105" s="4" t="n"/>
+      <c r="F105" s="4" t="inlineStr">
         <is>
           <t>hasElectrolyte-hasSolute-hasAdditive-hasConstituentB</t>
         </is>
       </c>
-      <c r="F105" s="4" t="n"/>
     </row>
     <row r="106">
       <c r="A106" s="16" t="inlineStr">
@@ -3210,12 +3210,12 @@
           <t>optional</t>
         </is>
       </c>
-      <c r="E106" s="16" t="inlineStr">
+      <c r="E106" s="16" t="n"/>
+      <c r="F106" s="16" t="inlineStr">
         <is>
           <t>hasElectrolyte-hasSolute-hasAdditive-hasConstituentB-hasMeasuredProperty-AmountConcentration</t>
         </is>
       </c>
-      <c r="F106" s="16" t="n"/>
     </row>
     <row r="107">
       <c r="A107" s="17" t="inlineStr">
@@ -3248,12 +3248,12 @@
           <t>optional</t>
         </is>
       </c>
-      <c r="E108" s="4" t="inlineStr">
+      <c r="E108" s="4" t="n"/>
+      <c r="F108" s="4" t="inlineStr">
         <is>
           <t>hasElectrolyte-hasMeasuredProperty-ElectrolyticConductivity</t>
         </is>
       </c>
-      <c r="F108" s="4" t="n"/>
     </row>
     <row r="109">
       <c r="A109" s="16" t="inlineStr">
@@ -3274,12 +3274,12 @@
           <t>optional</t>
         </is>
       </c>
-      <c r="E109" s="16" t="inlineStr">
+      <c r="E109" s="16" t="n"/>
+      <c r="F109" s="16" t="inlineStr">
         <is>
           <t>hasElectrolyte-hasMeasuredProperty-DynamicViscosity</t>
         </is>
       </c>
-      <c r="F109" s="16" t="n"/>
     </row>
     <row r="110">
       <c r="A110" s="4" t="inlineStr">
@@ -3300,12 +3300,12 @@
           <t>optional</t>
         </is>
       </c>
-      <c r="E110" s="4" t="inlineStr">
+      <c r="E110" s="4" t="n"/>
+      <c r="F110" s="4" t="inlineStr">
         <is>
           <t>hasElectrolyte-hasMeasuredProperty-Density</t>
         </is>
       </c>
-      <c r="F110" s="4" t="n"/>
     </row>
     <row r="111">
       <c r="A111" s="16" t="inlineStr">
@@ -3326,12 +3326,12 @@
           <t>optional</t>
         </is>
       </c>
-      <c r="E111" s="16" t="inlineStr">
+      <c r="E111" s="16" t="n"/>
+      <c r="F111" s="16" t="inlineStr">
         <is>
           <t>hasElectrolyte-hasMeasuredProperty-CelsiusTemperature</t>
         </is>
       </c>
-      <c r="F111" s="16" t="n"/>
     </row>
     <row r="112">
       <c r="A112" s="17" t="inlineStr">
@@ -3366,12 +3366,12 @@
           <t>optional</t>
         </is>
       </c>
-      <c r="E113" s="4" t="inlineStr">
+      <c r="E113" s="4" t="n"/>
+      <c r="F113" s="4" t="inlineStr">
         <is>
           <t>hasElectrolyte-schema:manufacturer</t>
         </is>
       </c>
-      <c r="F113" s="4" t="n"/>
     </row>
     <row r="114">
       <c r="A114" s="16" t="inlineStr">
@@ -3390,12 +3390,12 @@
           <t>optional</t>
         </is>
       </c>
-      <c r="E114" s="16" t="inlineStr">
+      <c r="E114" s="16" t="n"/>
+      <c r="F114" s="16" t="inlineStr">
         <is>
           <t>hasElectrolyte-schema:productID</t>
         </is>
       </c>
-      <c r="F114" s="16" t="n"/>
     </row>
     <row r="115">
       <c r="A115" s="4" t="inlineStr">
@@ -3414,12 +3414,12 @@
           <t>optional</t>
         </is>
       </c>
-      <c r="E115" s="4" t="inlineStr">
+      <c r="E115" s="4" t="n"/>
+      <c r="F115" s="4" t="inlineStr">
         <is>
           <t>hasElectrolyte-hasSolvent-hasConstituentA-schema:manufacturer</t>
         </is>
       </c>
-      <c r="F115" s="4" t="n"/>
     </row>
     <row r="116">
       <c r="A116" s="16" t="inlineStr">
@@ -3438,12 +3438,12 @@
           <t>optional</t>
         </is>
       </c>
-      <c r="E116" s="16" t="inlineStr">
+      <c r="E116" s="16" t="n"/>
+      <c r="F116" s="16" t="inlineStr">
         <is>
           <t>hasElectrolyte-hasSolvent-hasConstituentA-schema:productID</t>
         </is>
       </c>
-      <c r="F116" s="16" t="n"/>
     </row>
     <row r="117">
       <c r="A117" s="4" t="inlineStr">
@@ -3462,12 +3462,12 @@
           <t>optional</t>
         </is>
       </c>
-      <c r="E117" s="4" t="inlineStr">
+      <c r="E117" s="4" t="n"/>
+      <c r="F117" s="4" t="inlineStr">
         <is>
           <t>hasElectrolyte-hasSolvent-hasConstituentB-schema:manufacturer</t>
         </is>
       </c>
-      <c r="F117" s="4" t="n"/>
     </row>
     <row r="118">
       <c r="A118" s="16" t="inlineStr">
@@ -3486,12 +3486,12 @@
           <t>optional</t>
         </is>
       </c>
-      <c r="E118" s="16" t="inlineStr">
+      <c r="E118" s="16" t="n"/>
+      <c r="F118" s="16" t="inlineStr">
         <is>
           <t>hasElectrolyte-hasSolvent-hasConstituentB-schema:productID</t>
         </is>
       </c>
-      <c r="F118" s="16" t="n"/>
     </row>
     <row r="119">
       <c r="A119" s="4" t="inlineStr">
@@ -3510,12 +3510,12 @@
           <t>optional</t>
         </is>
       </c>
-      <c r="E119" s="4" t="inlineStr">
+      <c r="E119" s="4" t="n"/>
+      <c r="F119" s="4" t="inlineStr">
         <is>
           <t>hasElectrolyte-hasSolute-hasConstituentA-schema:manufacturer</t>
         </is>
       </c>
-      <c r="F119" s="4" t="n"/>
     </row>
     <row r="120">
       <c r="A120" s="16" t="inlineStr">
@@ -3534,12 +3534,12 @@
           <t>optional</t>
         </is>
       </c>
-      <c r="E120" s="16" t="inlineStr">
+      <c r="E120" s="16" t="n"/>
+      <c r="F120" s="16" t="inlineStr">
         <is>
           <t>hasElectrolyte-hasSolute-hasConstituentA-schema:productID</t>
         </is>
       </c>
-      <c r="F120" s="16" t="n"/>
     </row>
     <row r="121">
       <c r="A121" s="4" t="inlineStr">
@@ -3558,12 +3558,12 @@
           <t>optional</t>
         </is>
       </c>
-      <c r="E121" s="4" t="inlineStr">
+      <c r="E121" s="4" t="n"/>
+      <c r="F121" s="4" t="inlineStr">
         <is>
           <t>hasElectrolyte-hasSolute-hasConstituentB-schema:manufacturer</t>
         </is>
       </c>
-      <c r="F121" s="4" t="n"/>
     </row>
     <row r="122">
       <c r="A122" s="16" t="inlineStr">
@@ -3582,12 +3582,12 @@
           <t>optional</t>
         </is>
       </c>
-      <c r="E122" s="16" t="inlineStr">
+      <c r="E122" s="16" t="n"/>
+      <c r="F122" s="16" t="inlineStr">
         <is>
           <t>hasElectrolyte-hasSolute-hasConstituentB-schema:productID</t>
         </is>
       </c>
-      <c r="F122" s="16" t="n"/>
     </row>
     <row r="123">
       <c r="A123" s="4" t="inlineStr">
@@ -3606,12 +3606,12 @@
           <t>optional</t>
         </is>
       </c>
-      <c r="E123" s="4" t="inlineStr">
+      <c r="E123" s="4" t="n"/>
+      <c r="F123" s="4" t="inlineStr">
         <is>
           <t>hasElectrolyte-hasSolute-hasAdditive-hasConstituentA-schema:manufacturer</t>
         </is>
       </c>
-      <c r="F123" s="4" t="n"/>
     </row>
     <row r="124">
       <c r="A124" s="16" t="inlineStr">
@@ -3630,12 +3630,12 @@
           <t>optional</t>
         </is>
       </c>
-      <c r="E124" s="16" t="inlineStr">
+      <c r="E124" s="16" t="n"/>
+      <c r="F124" s="16" t="inlineStr">
         <is>
           <t>hasElectrolyte-hasSolute-hasAdditive-hasConstituentA-schema:productID</t>
         </is>
       </c>
-      <c r="F124" s="16" t="n"/>
     </row>
     <row r="125">
       <c r="A125" s="4" t="inlineStr">
@@ -3654,12 +3654,12 @@
           <t>optional</t>
         </is>
       </c>
-      <c r="E125" s="4" t="inlineStr">
+      <c r="E125" s="4" t="n"/>
+      <c r="F125" s="4" t="inlineStr">
         <is>
           <t>hasElectrolyte-hasSolute-hasAdditive-hasConstituentB-schema:manufacturer</t>
         </is>
       </c>
-      <c r="F125" s="4" t="n"/>
     </row>
     <row r="126">
       <c r="A126" s="16" t="inlineStr">
@@ -3678,12 +3678,12 @@
           <t>optional</t>
         </is>
       </c>
-      <c r="E126" s="16" t="inlineStr">
+      <c r="E126" s="16" t="n"/>
+      <c r="F126" s="16" t="inlineStr">
         <is>
           <t>hasElectrolyte-hasSolute-hasAdditive-hasConstituentB-schema:productID</t>
         </is>
       </c>
-      <c r="F126" s="16" t="n"/>
     </row>
     <row r="127">
       <c r="A127" s="2" t="inlineStr">
@@ -3718,12 +3718,12 @@
           <t>required</t>
         </is>
       </c>
-      <c r="E128" s="4" t="inlineStr">
+      <c r="E128" s="4" t="n"/>
+      <c r="F128" s="4" t="inlineStr">
         <is>
           <t>hasSeparator</t>
         </is>
       </c>
-      <c r="F128" s="4" t="n"/>
     </row>
     <row r="129">
       <c r="A129" s="5" t="inlineStr">
@@ -3744,12 +3744,12 @@
           <t>required</t>
         </is>
       </c>
-      <c r="E129" s="5" t="inlineStr">
+      <c r="E129" s="5" t="n"/>
+      <c r="F129" s="5" t="inlineStr">
         <is>
           <t>hasSeparator-hasMeasuredProperty-Thickness</t>
         </is>
       </c>
-      <c r="F129" s="5" t="n"/>
     </row>
     <row r="130">
       <c r="A130" s="18" t="inlineStr">
@@ -3782,12 +3782,12 @@
           <t>recommended</t>
         </is>
       </c>
-      <c r="E131" s="4" t="inlineStr">
+      <c r="E131" s="4" t="n"/>
+      <c r="F131" s="4" t="inlineStr">
         <is>
           <t>hasSeparator-hasMeasuredProperty-Porosity</t>
         </is>
       </c>
-      <c r="F131" s="4" t="n"/>
     </row>
     <row r="132">
       <c r="A132" s="5" t="inlineStr">
@@ -3808,12 +3808,12 @@
           <t>optional</t>
         </is>
       </c>
-      <c r="E132" s="5" t="inlineStr">
+      <c r="E132" s="5" t="n"/>
+      <c r="F132" s="5" t="inlineStr">
         <is>
           <t>hasSeparator-hasMeasuredProperty-Tortuosity</t>
         </is>
       </c>
-      <c r="F132" s="5" t="n"/>
     </row>
     <row r="133">
       <c r="A133" s="18" t="inlineStr">
@@ -3848,12 +3848,12 @@
           <t>optional</t>
         </is>
       </c>
-      <c r="E134" s="4" t="inlineStr">
+      <c r="E134" s="4" t="n"/>
+      <c r="F134" s="4" t="inlineStr">
         <is>
           <t>hasSeparator-schema:manufacturer</t>
         </is>
       </c>
-      <c r="F134" s="4" t="n"/>
     </row>
     <row r="135">
       <c r="A135" s="5" t="inlineStr">
@@ -3874,12 +3874,12 @@
           <t>optional</t>
         </is>
       </c>
-      <c r="E135" s="5" t="inlineStr">
+      <c r="E135" s="5" t="n"/>
+      <c r="F135" s="5" t="inlineStr">
         <is>
           <t>hasSeparator-schema:productID</t>
         </is>
       </c>
-      <c r="F135" s="5" t="n"/>
     </row>
     <row r="136">
       <c r="A136" s="2" t="inlineStr">
@@ -3914,12 +3914,12 @@
           <t>required</t>
         </is>
       </c>
-      <c r="E137" s="4" t="inlineStr">
+      <c r="E137" s="4" t="n"/>
+      <c r="F137" s="4" t="inlineStr">
         <is>
           <t>hasCase</t>
         </is>
       </c>
-      <c r="F137" s="4" t="n"/>
     </row>
     <row r="138">
       <c r="A138" s="5" t="inlineStr">
@@ -3942,12 +3942,12 @@
           <t>required</t>
         </is>
       </c>
-      <c r="E138" s="5" t="inlineStr">
+      <c r="E138" s="5" t="n"/>
+      <c r="F138" s="5" t="inlineStr">
         <is>
           <t>hasCase</t>
         </is>
       </c>
-      <c r="F138" s="5" t="n"/>
     </row>
     <row r="139">
       <c r="A139" s="4" t="inlineStr">
@@ -3970,12 +3970,12 @@
           <t>required</t>
         </is>
       </c>
-      <c r="E139" s="4" t="inlineStr">
+      <c r="E139" s="4" t="n"/>
+      <c r="F139" s="4" t="inlineStr">
         <is>
           <t>hasCase-hasComponentA-type|CellLid-hasCoating</t>
         </is>
       </c>
-      <c r="F139" s="4" t="n"/>
     </row>
     <row r="140">
       <c r="A140" s="5" t="inlineStr">
@@ -3998,12 +3998,12 @@
           <t>required</t>
         </is>
       </c>
-      <c r="E140" s="5" t="inlineStr">
+      <c r="E140" s="5" t="n"/>
+      <c r="F140" s="5" t="inlineStr">
         <is>
           <t>hasCase-hasComponentB-type|CellCan-hasCoating</t>
         </is>
       </c>
-      <c r="F140" s="5" t="n"/>
     </row>
     <row r="141">
       <c r="A141" s="4" t="inlineStr">
@@ -4024,12 +4024,12 @@
           <t>required</t>
         </is>
       </c>
-      <c r="E141" s="4" t="inlineStr">
+      <c r="E141" s="4" t="n"/>
+      <c r="F141" s="4" t="inlineStr">
         <is>
           <t>hasComponentA-type|Spring-hasMeasuredProperty-Diameter</t>
         </is>
       </c>
-      <c r="F141" s="4" t="n"/>
     </row>
     <row r="142">
       <c r="A142" s="5" t="inlineStr">
@@ -4050,12 +4050,12 @@
           <t>required</t>
         </is>
       </c>
-      <c r="E142" s="5" t="inlineStr">
+      <c r="E142" s="5" t="n"/>
+      <c r="F142" s="5" t="inlineStr">
         <is>
           <t>hasComponentA-type|Spring-hasMeasuredProperty-Thickness</t>
         </is>
       </c>
-      <c r="F142" s="5" t="n"/>
     </row>
     <row r="143">
       <c r="A143" s="4" t="inlineStr">
@@ -4076,12 +4076,12 @@
           <t>required</t>
         </is>
       </c>
-      <c r="E143" s="4" t="inlineStr">
+      <c r="E143" s="4" t="n"/>
+      <c r="F143" s="4" t="inlineStr">
         <is>
           <t>hasComponentB-type|Spacer-hasMeasuredProperty-Diameter</t>
         </is>
       </c>
-      <c r="F143" s="4" t="n"/>
     </row>
     <row r="144">
       <c r="A144" s="5" t="inlineStr">
@@ -4102,12 +4102,12 @@
           <t>required</t>
         </is>
       </c>
-      <c r="E144" s="5" t="inlineStr">
+      <c r="E144" s="5" t="n"/>
+      <c r="F144" s="5" t="inlineStr">
         <is>
           <t>hasComponentB-type|Spacer-hasMeasuredProperty-Thickness</t>
         </is>
       </c>
-      <c r="F144" s="5" t="n"/>
     </row>
     <row r="145">
       <c r="A145" s="4" t="inlineStr">
@@ -4128,12 +4128,12 @@
           <t>required</t>
         </is>
       </c>
-      <c r="E145" s="4" t="inlineStr">
+      <c r="E145" s="4" t="n"/>
+      <c r="F145" s="4" t="inlineStr">
         <is>
           <t>hasPositiveElectrode-hasMeasuredProperty-Diameter</t>
         </is>
       </c>
-      <c r="F145" s="4" t="n"/>
     </row>
     <row r="146">
       <c r="A146" s="5" t="inlineStr">
@@ -4154,12 +4154,12 @@
           <t>recommended</t>
         </is>
       </c>
-      <c r="E146" s="5" t="inlineStr">
+      <c r="E146" s="5" t="n"/>
+      <c r="F146" s="5" t="inlineStr">
         <is>
           <t>hasNegativeElectrode-hasMeasuredProperty-Diameter</t>
         </is>
       </c>
-      <c r="F146" s="5" t="n"/>
     </row>
     <row r="147">
       <c r="A147" s="4" t="inlineStr">
@@ -4180,12 +4180,12 @@
           <t>recommended</t>
         </is>
       </c>
-      <c r="E147" s="4" t="inlineStr">
+      <c r="E147" s="4" t="n"/>
+      <c r="F147" s="4" t="inlineStr">
         <is>
           <t>hasSeparator-hasMeasuredProperty-Diameter</t>
         </is>
       </c>
-      <c r="F147" s="4" t="n"/>
     </row>
     <row r="148">
       <c r="A148" s="5" t="inlineStr">
@@ -4206,12 +4206,12 @@
           <t>required</t>
         </is>
       </c>
-      <c r="E148" s="5" t="inlineStr">
+      <c r="E148" s="5" t="n"/>
+      <c r="F148" s="5" t="inlineStr">
         <is>
           <t>hasElectrolyte-hasMeasuredProperty-Volume</t>
         </is>
       </c>
-      <c r="F148" s="5" t="n"/>
     </row>
     <row r="149">
       <c r="A149" s="4" t="inlineStr">
@@ -4234,12 +4234,12 @@
           <t>optional</t>
         </is>
       </c>
-      <c r="E149" s="4" t="inlineStr">
+      <c r="E149" s="4" t="n"/>
+      <c r="F149" s="4" t="inlineStr">
         <is>
           <t>rdfs:comment</t>
         </is>
       </c>
-      <c r="F149" s="4" t="n"/>
     </row>
     <row r="150">
       <c r="A150" s="18" t="inlineStr">
@@ -4274,12 +4274,12 @@
           <t>optional</t>
         </is>
       </c>
-      <c r="E151" s="4" t="inlineStr">
+      <c r="E151" s="4" t="n"/>
+      <c r="F151" s="4" t="inlineStr">
         <is>
           <t>hasCase-schema:manufacturer</t>
         </is>
       </c>
-      <c r="F151" s="4" t="n"/>
     </row>
     <row r="152">
       <c r="A152" s="5" t="inlineStr">
@@ -4302,12 +4302,12 @@
           <t>optional</t>
         </is>
       </c>
-      <c r="E152" s="5" t="inlineStr">
+      <c r="E152" s="5" t="n"/>
+      <c r="F152" s="5" t="inlineStr">
         <is>
           <t>hasCase-schema:productID</t>
         </is>
       </c>
-      <c r="F152" s="5" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Remove unnecessary prefixes in all templates
</commit_message>
<xml_diff>
--- a/test/data/coincell_excel_schema.xlsx
+++ b/test/data/coincell_excel_schema.xlsx
@@ -863,7 +863,7 @@
       </c>
       <c r="B12" s="5" t="inlineStr">
         <is>
-          <t>1.1.17</t>
+          <t>1.1.18</t>
         </is>
       </c>
       <c r="C12" s="5" t="inlineStr">
@@ -5001,7 +5001,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>unit:MilliM</t>
+          <t>MilliMetre</t>
         </is>
       </c>
     </row>
@@ -5025,7 +5025,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>unit:MilliGM-PER-CentiM2</t>
+          <t>MilliGramPerSquareCentiMetre</t>
         </is>
       </c>
     </row>
@@ -5049,7 +5049,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>unit:MilliGM</t>
+          <t>MilliGram</t>
         </is>
       </c>
     </row>
@@ -5073,7 +5073,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>unit:MOL</t>
+          <t>Mole</t>
         </is>
       </c>
     </row>
@@ -5097,7 +5097,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>emmo:MicroMetre</t>
+          <t>MicroMetre</t>
         </is>
       </c>
     </row>
@@ -5109,7 +5109,7 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>unit:V</t>
+          <t>Volt</t>
         </is>
       </c>
     </row>
@@ -5121,7 +5121,7 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>emmo:MilliAmperePerSquareCentiMetre</t>
+          <t>MilliAmperePerSquareCentiMetre</t>
         </is>
       </c>
     </row>
@@ -5145,7 +5145,7 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>unit:MOL-PER-L</t>
+          <t>MolePerCubicDeciMetre</t>
         </is>
       </c>
     </row>
@@ -5157,7 +5157,7 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>unit:MilliS-PER-CentiM</t>
+          <t>MilliSiemensPerCentiMetre</t>
         </is>
       </c>
     </row>
@@ -5169,7 +5169,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>unit:MilliPA-SEC</t>
+          <t>MilliPascalSecond</t>
         </is>
       </c>
     </row>
@@ -5181,7 +5181,7 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>emmo:GramPerCubicCentiMetre</t>
+          <t>GramPerCubicCentiMetre</t>
         </is>
       </c>
     </row>
@@ -5193,7 +5193,7 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>emmo:CelsiusTemperature</t>
+          <t>DegreeCelsius</t>
         </is>
       </c>
     </row>
@@ -5205,7 +5205,7 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>emmo:UnitOne</t>
+          <t>UnitOne</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update literals, remove unnecessary prefixes (#96)
* Automatically populate string literal values

* Update context

* Override "hasMeasurementUnit" to "@vocab", so values like "Volt" are expanded as IRIs not string literals

* Add warning for unnecessary prefixes

* Remove unnecessary prefixes in all templates
</commit_message>
<xml_diff>
--- a/test/data/coincell_excel_schema.xlsx
+++ b/test/data/coincell_excel_schema.xlsx
@@ -863,7 +863,7 @@
       </c>
       <c r="B12" s="5" t="inlineStr">
         <is>
-          <t>1.1.17</t>
+          <t>1.1.18</t>
         </is>
       </c>
       <c r="C12" s="5" t="inlineStr">
@@ -5001,7 +5001,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>unit:MilliM</t>
+          <t>MilliMetre</t>
         </is>
       </c>
     </row>
@@ -5025,7 +5025,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>unit:MilliGM-PER-CentiM2</t>
+          <t>MilliGramPerSquareCentiMetre</t>
         </is>
       </c>
     </row>
@@ -5049,7 +5049,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>unit:MilliGM</t>
+          <t>MilliGram</t>
         </is>
       </c>
     </row>
@@ -5073,7 +5073,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>unit:MOL</t>
+          <t>Mole</t>
         </is>
       </c>
     </row>
@@ -5097,7 +5097,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>emmo:MicroMetre</t>
+          <t>MicroMetre</t>
         </is>
       </c>
     </row>
@@ -5109,7 +5109,7 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>unit:V</t>
+          <t>Volt</t>
         </is>
       </c>
     </row>
@@ -5121,7 +5121,7 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>emmo:MilliAmperePerSquareCentiMetre</t>
+          <t>MilliAmperePerSquareCentiMetre</t>
         </is>
       </c>
     </row>
@@ -5145,7 +5145,7 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>unit:MOL-PER-L</t>
+          <t>MolePerCubicDeciMetre</t>
         </is>
       </c>
     </row>
@@ -5157,7 +5157,7 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>unit:MilliS-PER-CentiM</t>
+          <t>MilliSiemensPerCentiMetre</t>
         </is>
       </c>
     </row>
@@ -5169,7 +5169,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>unit:MilliPA-SEC</t>
+          <t>MilliPascalSecond</t>
         </is>
       </c>
     </row>
@@ -5181,7 +5181,7 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>emmo:GramPerCubicCentiMetre</t>
+          <t>GramPerCubicCentiMetre</t>
         </is>
       </c>
     </row>
@@ -5193,7 +5193,7 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>emmo:CelsiusTemperature</t>
+          <t>DegreeCelsius</t>
         </is>
       </c>
     </row>
@@ -5205,7 +5205,7 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>emmo:UnitOne</t>
+          <t>UnitOne</t>
         </is>
       </c>
     </row>

</xml_diff>